<commit_message>
Updated Direct GRN And Sales invoices Test Data And locators
Updated Direct GRN And Sales invoices Test Data And locators
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4278" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4118" uniqueCount="197">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -607,37 +607,13 @@
     <t>184.24408</t>
   </si>
   <si>
-    <t>TVS-RM-KDK-20</t>
-  </si>
-  <si>
-    <t>685</t>
-  </si>
-  <si>
-    <t>147.08442</t>
-  </si>
-  <si>
     <t>189.55072</t>
   </si>
   <si>
     <t>190.42571</t>
   </si>
   <si>
-    <t>14048</t>
-  </si>
-  <si>
-    <t>120.68321</t>
-  </si>
-  <si>
     <t>57.048</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>38.334</t>
-  </si>
-  <si>
-    <t>56.89696</t>
   </si>
   <si>
     <t>71.668</t>
@@ -646,130 +622,7 @@
     <t>56.96721</t>
   </si>
   <si>
-    <t>14050</t>
-  </si>
-  <si>
-    <t>120.70622</t>
-  </si>
-  <si>
-    <t>14052</t>
-  </si>
-  <si>
-    <t>120.72922</t>
-  </si>
-  <si>
-    <t>14054</t>
-  </si>
-  <si>
-    <t>120.75222</t>
-  </si>
-  <si>
-    <t>14056</t>
-  </si>
-  <si>
-    <t>120.77521</t>
-  </si>
-  <si>
-    <t>14058</t>
-  </si>
-  <si>
-    <t>120.79819</t>
-  </si>
-  <si>
-    <t>14060</t>
-  </si>
-  <si>
-    <t>120.82117</t>
-  </si>
-  <si>
-    <t>14062</t>
-  </si>
-  <si>
-    <t>120.84414</t>
-  </si>
-  <si>
-    <t>14064</t>
-  </si>
-  <si>
-    <t>120.8671</t>
-  </si>
-  <si>
-    <t>14066</t>
-  </si>
-  <si>
-    <t>120.89006</t>
-  </si>
-  <si>
-    <t>14070</t>
-  </si>
-  <si>
-    <t>120.93595</t>
-  </si>
-  <si>
-    <t>14072</t>
-  </si>
-  <si>
-    <t>120.95889</t>
-  </si>
-  <si>
-    <t>14074</t>
-  </si>
-  <si>
-    <t>120.98182</t>
-  </si>
-  <si>
-    <t>14076</t>
-  </si>
-  <si>
-    <t>121.00475</t>
-  </si>
-  <si>
-    <t>14078</t>
-  </si>
-  <si>
-    <t>121.02767</t>
-  </si>
-  <si>
-    <t>14080</t>
-  </si>
-  <si>
-    <t>121.05058</t>
-  </si>
-  <si>
-    <t>14082</t>
-  </si>
-  <si>
-    <t>121.07349</t>
-  </si>
-  <si>
-    <t>14084</t>
-  </si>
-  <si>
-    <t>121.09639</t>
-  </si>
-  <si>
-    <t>14086</t>
-  </si>
-  <si>
-    <t>121.11928</t>
-  </si>
-  <si>
-    <t>14088</t>
-  </si>
-  <si>
-    <t>121.14217</t>
-  </si>
-  <si>
     <t>14090</t>
-  </si>
-  <si>
-    <t>121.19751</t>
-  </si>
-  <si>
-    <t>689</t>
-  </si>
-  <si>
-    <t>146.93409</t>
   </si>
   <si>
     <t>121.22038</t>
@@ -779,6 +632,15 @@
   </si>
   <si>
     <t>146.85967</t>
+  </si>
+  <si>
+    <t>TVS-SER-10001-PriceList</t>
+  </si>
+  <si>
+    <t>TVS-SER-10001-RateContract</t>
+  </si>
+  <si>
+    <t>TVS-RM-KDK-101</t>
   </si>
 </sst>
 </file>
@@ -1565,7 +1427,7 @@
   <dimension ref="A8:BR37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="27.28515625"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:70" ht="15.75" thickBot="1"/>
@@ -1733,10 +1595,10 @@
       <c r="AT9" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU9" t="s" s="0">
+      <c r="AU9" t="s">
         <v>127</v>
       </c>
-      <c r="AV9" t="s" s="0">
+      <c r="AV9" t="s">
         <v>143</v>
       </c>
       <c r="AW9" s="48">
@@ -1777,10 +1639,10 @@
       <c r="BL9" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM9" t="s" s="0">
+      <c r="BM9" t="s">
         <v>146</v>
       </c>
-      <c r="BN9" t="s" s="0">
+      <c r="BN9" t="s">
         <v>147</v>
       </c>
       <c r="BO9" s="48" t="e">
@@ -1952,20 +1814,20 @@
       <c r="AQ15" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR15" t="e" s="0">
+      <c r="AR15" t="e">
         <f>ROUND(AN15+AO15+AP15,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS15" t="s" s="0">
+      <c r="AS15" t="s">
         <v>107</v>
       </c>
       <c r="AT15" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU15" t="s" s="0">
+      <c r="AU15" t="s">
         <v>131</v>
       </c>
-      <c r="AV15" t="s" s="0">
+      <c r="AV15" t="s">
         <v>149</v>
       </c>
       <c r="AW15" s="48">
@@ -2004,10 +1866,10 @@
       <c r="BL15" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM15" t="s" s="0">
+      <c r="BM15" t="s">
         <v>149</v>
       </c>
-      <c r="BN15" t="s" s="0">
+      <c r="BN15" t="s">
         <v>150</v>
       </c>
       <c r="BO15" s="48" t="e">
@@ -2177,20 +2039,20 @@
       <c r="AQ16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR16" s="0">
+      <c r="AR16">
         <f>ROUND(AN16+AO16+AP16,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS16" t="s" s="0">
+      <c r="AS16" t="s">
         <v>107</v>
       </c>
       <c r="AT16" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU16" t="s" s="0">
+      <c r="AU16" t="s">
         <v>135</v>
       </c>
-      <c r="AV16" t="s" s="0">
+      <c r="AV16" t="s">
         <v>136</v>
       </c>
       <c r="AW16" s="48">
@@ -2229,10 +2091,10 @@
       <c r="BL16" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM16" t="s" s="0">
+      <c r="BM16" t="s">
         <v>134</v>
       </c>
-      <c r="BN16" t="s" s="0">
+      <c r="BN16" t="s">
         <v>133</v>
       </c>
       <c r="BO16" s="48">
@@ -2402,20 +2264,20 @@
       <c r="AQ17" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR17" s="0">
+      <c r="AR17">
         <f>ROUND(AN17+AO17+AP17,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS17" t="s" s="0">
+      <c r="AS17" t="s">
         <v>107</v>
       </c>
       <c r="AT17" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU17" t="s" s="0">
+      <c r="AU17" t="s">
         <v>108</v>
       </c>
-      <c r="AV17" t="s" s="0">
+      <c r="AV17" t="s">
         <v>132</v>
       </c>
       <c r="AW17" s="48">
@@ -2621,20 +2483,20 @@
       <c r="AQ18" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR18" s="0">
+      <c r="AR18">
         <f>ROUND(AN18+AO18+AP18,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS18" t="s" s="0">
+      <c r="AS18" t="s">
         <v>107</v>
       </c>
       <c r="AT18" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU18" t="s" s="0">
+      <c r="AU18" t="s">
         <v>130</v>
       </c>
-      <c r="AV18" t="s" s="0">
+      <c r="AV18" t="s">
         <v>137</v>
       </c>
       <c r="AW18" s="48">
@@ -2673,10 +2535,10 @@
       <c r="BL18" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM18" t="s" s="0">
+      <c r="BM18" t="s">
         <v>153</v>
       </c>
-      <c r="BN18" t="s" s="0">
+      <c r="BN18" t="s">
         <v>152</v>
       </c>
       <c r="BO18" s="48">
@@ -2847,20 +2709,20 @@
       <c r="AQ20" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR20" t="e" s="0">
+      <c r="AR20" t="e">
         <f>ROUND(AN20+AO20+AP20,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS20" t="s" s="0">
+      <c r="AS20" t="s">
         <v>107</v>
       </c>
       <c r="AT20" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU20" t="s" s="0">
+      <c r="AU20" t="s">
         <v>155</v>
       </c>
-      <c r="AV20" t="s" s="0">
+      <c r="AV20" t="s">
         <v>156</v>
       </c>
       <c r="AW20" s="48">
@@ -2899,10 +2761,10 @@
       <c r="BL20" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM20" t="s" s="0">
+      <c r="BM20" t="s">
         <v>156</v>
       </c>
-      <c r="BN20" t="s" s="0">
+      <c r="BN20" t="s">
         <v>127</v>
       </c>
       <c r="BO20" s="48" t="e">
@@ -3072,20 +2934,20 @@
       <c r="AQ21" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR21" t="e" s="0">
+      <c r="AR21" t="e">
         <f t="shared" ref="AR21:AR23" si="30">ROUND(AN21+AO21+AP21,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS21" t="s" s="0">
+      <c r="AS21" t="s">
         <v>107</v>
       </c>
       <c r="AT21" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU21" t="s" s="0">
+      <c r="AU21" t="s">
         <v>131</v>
       </c>
-      <c r="AV21" t="s" s="0">
+      <c r="AV21" t="s">
         <v>157</v>
       </c>
       <c r="AW21" s="48">
@@ -3124,10 +2986,10 @@
       <c r="BL21" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM21" t="s" s="0">
+      <c r="BM21" t="s">
         <v>108</v>
       </c>
-      <c r="BN21" t="s" s="0">
+      <c r="BN21" t="s">
         <v>108</v>
       </c>
       <c r="BO21" s="48" t="e">
@@ -3297,20 +3159,20 @@
       <c r="AQ22" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR22" t="e" s="0">
+      <c r="AR22" t="e">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS22" t="s" s="0">
+      <c r="AS22" t="s">
         <v>107</v>
       </c>
       <c r="AT22" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU22" t="s" s="0">
+      <c r="AU22" t="s">
         <v>158</v>
       </c>
-      <c r="AV22" t="s" s="0">
+      <c r="AV22" t="s">
         <v>159</v>
       </c>
       <c r="AW22" s="48">
@@ -3349,10 +3211,10 @@
       <c r="BL22" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM22" t="s" s="0">
+      <c r="BM22" t="s">
         <v>108</v>
       </c>
-      <c r="BN22" t="s" s="0">
+      <c r="BN22" t="s">
         <v>108</v>
       </c>
       <c r="BO22" s="48" t="e">
@@ -3522,20 +3384,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" t="e" s="0">
+      <c r="AR23" t="e">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>160</v>
       </c>
       <c r="AW23" s="48">
@@ -3574,10 +3436,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48" t="e">
@@ -3634,14 +3496,14 @@
       <c r="F31" s="46">
         <v>2</v>
       </c>
-      <c r="G31" t="s" s="0">
+      <c r="G31" t="s">
         <v>128</v>
       </c>
       <c r="H31" s="46">
         <f>F31*G31</f>
         <v>600</v>
       </c>
-      <c r="I31" t="s" s="0">
+      <c r="I31" t="s">
         <v>127</v>
       </c>
       <c r="J31" s="46">
@@ -3769,20 +3631,20 @@
       <c r="AQ31" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR31" s="0">
+      <c r="AR31">
         <f>ROUND(AN31+AO31+AP31,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS31" t="s" s="0">
+      <c r="AS31" t="s">
         <v>107</v>
       </c>
       <c r="AT31" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU31" t="s" s="0">
+      <c r="AU31" t="s">
         <v>162</v>
       </c>
-      <c r="AV31" t="s" s="0">
+      <c r="AV31" t="s">
         <v>170</v>
       </c>
       <c r="AW31" s="48">
@@ -3821,10 +3683,10 @@
       <c r="BL31" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM31" t="s" s="0">
+      <c r="BM31" t="s">
         <v>108</v>
       </c>
-      <c r="BN31" t="s" s="0">
+      <c r="BN31" t="s">
         <v>108</v>
       </c>
       <c r="BO31" s="48">
@@ -3859,14 +3721,14 @@
       <c r="F32" s="46">
         <v>2</v>
       </c>
-      <c r="G32" t="s" s="0">
+      <c r="G32" t="s">
         <v>129</v>
       </c>
       <c r="H32" s="46">
         <f>F32*G32</f>
         <v>800</v>
       </c>
-      <c r="I32" t="s" s="0">
+      <c r="I32" t="s">
         <v>127</v>
       </c>
       <c r="J32" s="46">
@@ -3994,20 +3856,20 @@
       <c r="AQ32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR32" s="0">
+      <c r="AR32">
         <f>ROUND(AN32+AO32+AP32,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS32" t="s" s="0">
+      <c r="AS32" t="s">
         <v>107</v>
       </c>
       <c r="AT32" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU32" t="s" s="0">
+      <c r="AU32" t="s">
         <v>171</v>
       </c>
-      <c r="AV32" t="s" s="0">
+      <c r="AV32" t="s">
         <v>172</v>
       </c>
       <c r="AW32" s="48">
@@ -4046,10 +3908,10 @@
       <c r="BL32" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM32" t="s" s="0">
+      <c r="BM32" t="s">
         <v>108</v>
       </c>
-      <c r="BN32" t="s" s="0">
+      <c r="BN32" t="s">
         <v>108</v>
       </c>
       <c r="BO32" s="48">
@@ -4084,14 +3946,14 @@
       <c r="F33" s="46">
         <v>2</v>
       </c>
-      <c r="G33" t="s" s="0">
+      <c r="G33" t="s">
         <v>161</v>
       </c>
       <c r="H33" s="46">
         <f>F33*G33</f>
         <v>1000</v>
       </c>
-      <c r="I33" t="s" s="0">
+      <c r="I33" t="s">
         <v>127</v>
       </c>
       <c r="J33" s="46">
@@ -4219,20 +4081,20 @@
       <c r="AQ33" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR33" s="0">
+      <c r="AR33">
         <f>ROUND(AN33+AO33+AP33,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS33" t="s" s="0">
+      <c r="AS33" t="s">
         <v>107</v>
       </c>
       <c r="AT33" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU33" t="s" s="0">
+      <c r="AU33" t="s">
         <v>108</v>
       </c>
-      <c r="AV33" t="s" s="0">
+      <c r="AV33" t="s">
         <v>173</v>
       </c>
       <c r="AW33" s="48">
@@ -4271,10 +4133,10 @@
       <c r="BL33" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM33" t="s" s="0">
+      <c r="BM33" t="s">
         <v>108</v>
       </c>
-      <c r="BN33" t="s" s="0">
+      <c r="BN33" t="s">
         <v>108</v>
       </c>
       <c r="BO33" s="48">
@@ -4310,14 +4172,14 @@
       <c r="F35" s="46">
         <v>2</v>
       </c>
-      <c r="G35" t="s" s="0">
+      <c r="G35" t="s">
         <v>128</v>
       </c>
       <c r="H35" s="46">
         <f>F35*G35</f>
         <v>600</v>
       </c>
-      <c r="I35" t="s" s="0">
+      <c r="I35" t="s">
         <v>127</v>
       </c>
       <c r="J35" s="46">
@@ -4445,20 +4307,20 @@
       <c r="AQ35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR35" s="0">
+      <c r="AR35">
         <f>ROUND(AN35+AO35+AP35,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS35" t="s" s="0">
+      <c r="AS35" t="s">
         <v>107</v>
       </c>
       <c r="AT35" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU35" t="s" s="0">
+      <c r="AU35" t="s">
         <v>174</v>
       </c>
-      <c r="AV35" t="s" s="0">
+      <c r="AV35" t="s">
         <v>175</v>
       </c>
       <c r="AW35" s="48">
@@ -4497,10 +4359,10 @@
       <c r="BL35" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM35" t="s" s="0">
+      <c r="BM35" t="s">
         <v>108</v>
       </c>
-      <c r="BN35" t="s" s="0">
+      <c r="BN35" t="s">
         <v>108</v>
       </c>
       <c r="BO35" s="48">
@@ -4535,14 +4397,14 @@
       <c r="F36" s="46">
         <v>2</v>
       </c>
-      <c r="G36" t="s" s="0">
+      <c r="G36" t="s">
         <v>129</v>
       </c>
       <c r="H36" s="46">
         <f>F36*G36</f>
         <v>800</v>
       </c>
-      <c r="I36" t="s" s="0">
+      <c r="I36" t="s">
         <v>127</v>
       </c>
       <c r="J36" s="46">
@@ -4670,20 +4532,20 @@
       <c r="AQ36" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR36" s="0">
+      <c r="AR36">
         <f>ROUND(AN36+AO36+AP36,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS36" t="s" s="0">
+      <c r="AS36" t="s">
         <v>107</v>
       </c>
       <c r="AT36" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU36" t="s" s="0">
+      <c r="AU36" t="s">
         <v>176</v>
       </c>
-      <c r="AV36" t="s" s="0">
+      <c r="AV36" t="s">
         <v>177</v>
       </c>
       <c r="AW36" s="48">
@@ -4722,10 +4584,10 @@
       <c r="BL36" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM36" t="s" s="0">
+      <c r="BM36" t="s">
         <v>108</v>
       </c>
-      <c r="BN36" t="s" s="0">
+      <c r="BN36" t="s">
         <v>108</v>
       </c>
       <c r="BO36" s="48">
@@ -4760,14 +4622,14 @@
       <c r="F37" s="46">
         <v>2</v>
       </c>
-      <c r="G37" t="s" s="0">
+      <c r="G37" t="s">
         <v>161</v>
       </c>
       <c r="H37" s="46">
         <f>F37*G37</f>
         <v>1000</v>
       </c>
-      <c r="I37" t="s" s="0">
+      <c r="I37" t="s">
         <v>127</v>
       </c>
       <c r="J37" s="46">
@@ -4895,20 +4757,20 @@
       <c r="AQ37" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR37" s="0">
+      <c r="AR37">
         <f>ROUND(AN37+AO37+AP37,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS37" t="s" s="0">
+      <c r="AS37" t="s">
         <v>107</v>
       </c>
       <c r="AT37" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU37" t="s" s="0">
+      <c r="AU37" t="s">
         <v>108</v>
       </c>
-      <c r="AV37" t="s" s="0">
+      <c r="AV37" t="s">
         <v>173</v>
       </c>
       <c r="AW37" s="48">
@@ -4947,10 +4809,10 @@
       <c r="BL37" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM37" t="s" s="0">
+      <c r="BM37" t="s">
         <v>108</v>
       </c>
-      <c r="BN37" t="s" s="0">
+      <c r="BN37" t="s">
         <v>108</v>
       </c>
       <c r="BO37" s="48">
@@ -4976,34 +4838,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -6515,10 +6377,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>118</v>
+        <v>196</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>118</v>
+        <v>196</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -6529,14 +6391,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -6664,20 +6526,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -6716,10 +6578,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -6894,32 +6756,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -8445,14 +8307,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -8580,11 +8442,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -8795,34 +8657,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -10334,10 +10196,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -10348,14 +10210,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -10483,20 +10345,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -10535,10 +10397,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -10713,32 +10575,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -12250,10 +12112,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -12264,14 +12126,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -12399,11 +12261,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -12614,34 +12476,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -14153,10 +14015,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -14167,14 +14029,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -14302,20 +14164,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -14354,10 +14216,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -14532,32 +14394,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -16069,10 +15931,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -16083,14 +15945,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -16218,11 +16080,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -16433,34 +16295,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -18121,20 +17983,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>178</v>
       </c>
       <c r="AW23" s="48">
@@ -18173,10 +18035,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>178</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>179</v>
       </c>
       <c r="BO23" s="48">
@@ -18348,34 +18210,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -20036,20 +19898,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>131</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -20088,10 +19950,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>150</v>
       </c>
       <c r="BO23" s="48">
@@ -20263,32 +20125,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -21814,14 +21676,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -21949,11 +21811,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -22164,34 +22026,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -23717,14 +23579,14 @@
       <c r="F23" s="46">
         <v>50</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>1000</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -23852,21 +23714,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>57.048000000000002</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>192</v>
+      <c r="AV23" t="s">
+        <v>187</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -23904,11 +23766,11 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>197</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>196</v>
+      <c r="BM23" t="s">
+        <v>189</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>188</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -24079,34 +23941,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -25618,10 +25480,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>11</v>
+        <v>196</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -25767,21 +25629,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
-        <v>236</v>
-      </c>
-      <c r="AV23" t="s" s="0">
-        <v>240</v>
+      <c r="AU23" t="s">
+        <v>190</v>
+      </c>
+      <c r="AV23" t="s">
+        <v>191</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -25819,11 +25681,11 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>242</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>241</v>
+      <c r="BM23" t="s">
+        <v>193</v>
+      </c>
+      <c r="BN23" t="s">
+        <v>192</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -25995,34 +25857,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -27548,14 +27410,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>60</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -27683,20 +27545,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>55.89</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>180</v>
       </c>
       <c r="AW23" s="48">
@@ -27735,10 +27597,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>180</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>130</v>
       </c>
       <c r="BO23" s="48">
@@ -27910,32 +27772,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -29461,14 +29323,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -29596,11 +29458,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -29811,34 +29673,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -31364,14 +31226,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>60</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -31499,20 +31361,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>55.89</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>181</v>
       </c>
       <c r="AW23" s="48">
@@ -31551,10 +31413,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>181</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>150</v>
       </c>
       <c r="BO23" s="48">
@@ -31729,34 +31591,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -33282,14 +33144,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>60</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -33417,20 +33279,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>56.46</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>181</v>
       </c>
       <c r="AW23" s="48">
@@ -33469,10 +33331,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>181</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>158</v>
       </c>
       <c r="BO23" s="48">
@@ -33647,32 +33509,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -35198,14 +35060,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -35333,11 +35195,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -35548,32 +35410,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -37085,10 +36947,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>154</v>
+        <v>196</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>154</v>
+        <v>196</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -37234,20 +37096,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>131</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -37286,10 +37148,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>182</v>
       </c>
       <c r="BO23" s="48">
@@ -37464,32 +37326,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -39150,11 +39012,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -39365,34 +39227,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -40918,14 +40780,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -41053,21 +40915,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>155</v>
       </c>
-      <c r="AV23" t="s" s="0">
-        <v>188</v>
+      <c r="AV23" t="s">
+        <v>185</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -41105,10 +40967,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
-        <v>189</v>
-      </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BM23" t="s">
+        <v>186</v>
+      </c>
+      <c r="BN23" t="s">
         <v>150</v>
       </c>
       <c r="BO23" s="48">
@@ -41280,32 +41142,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -42817,10 +42679,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>117</v>
+        <v>195</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -42831,14 +42693,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -42966,11 +42828,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -43181,34 +43043,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -44734,14 +44596,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -44869,20 +44731,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>158</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>183</v>
       </c>
       <c r="AW23" s="48">
@@ -44921,10 +44783,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>184</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>131</v>
       </c>
       <c r="BO23" s="48">
@@ -45100,32 +44962,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -46637,10 +46499,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>117</v>
+        <v>194</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -46651,14 +46513,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -46786,11 +46648,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -46993,6 +46855,7 @@
     <mergeCell ref="A1:AC1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -47001,34 +46864,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -48540,10 +48403,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>118</v>
+        <v>196</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>118</v>
+        <v>196</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -48554,14 +48417,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -48689,20 +48552,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>132</v>
       </c>
       <c r="AW23" s="48">
@@ -48741,10 +48604,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48">

</xml_diff>

<commit_message>
Updated Username And Password For All Modules
Updated Username And Password For All Modules Then Locator Fixes For The SCO And Sales Invoice Screens
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" activeTab="4"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="21" activeTab="23"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4122" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4118" uniqueCount="196">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -1424,7 +1424,7 @@
   <dimension ref="A8:BR37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="27.28515625"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:70" ht="15.75" thickBot="1"/>
@@ -1592,10 +1592,10 @@
       <c r="AT9" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU9" t="s" s="0">
+      <c r="AU9" t="s">
         <v>127</v>
       </c>
-      <c r="AV9" t="s" s="0">
+      <c r="AV9" t="s">
         <v>143</v>
       </c>
       <c r="AW9" s="48">
@@ -1636,10 +1636,10 @@
       <c r="BL9" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM9" t="s" s="0">
+      <c r="BM9" t="s">
         <v>146</v>
       </c>
-      <c r="BN9" t="s" s="0">
+      <c r="BN9" t="s">
         <v>147</v>
       </c>
       <c r="BO9" s="48" t="e">
@@ -1811,20 +1811,20 @@
       <c r="AQ15" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR15" t="e" s="0">
+      <c r="AR15" t="e">
         <f>ROUND(AN15+AO15+AP15,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS15" t="s" s="0">
+      <c r="AS15" t="s">
         <v>107</v>
       </c>
       <c r="AT15" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU15" t="s" s="0">
+      <c r="AU15" t="s">
         <v>131</v>
       </c>
-      <c r="AV15" t="s" s="0">
+      <c r="AV15" t="s">
         <v>149</v>
       </c>
       <c r="AW15" s="48">
@@ -1863,10 +1863,10 @@
       <c r="BL15" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM15" t="s" s="0">
+      <c r="BM15" t="s">
         <v>149</v>
       </c>
-      <c r="BN15" t="s" s="0">
+      <c r="BN15" t="s">
         <v>150</v>
       </c>
       <c r="BO15" s="48" t="e">
@@ -2036,20 +2036,20 @@
       <c r="AQ16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR16" s="0">
+      <c r="AR16">
         <f>ROUND(AN16+AO16+AP16,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS16" t="s" s="0">
+      <c r="AS16" t="s">
         <v>107</v>
       </c>
       <c r="AT16" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU16" t="s" s="0">
+      <c r="AU16" t="s">
         <v>135</v>
       </c>
-      <c r="AV16" t="s" s="0">
+      <c r="AV16" t="s">
         <v>136</v>
       </c>
       <c r="AW16" s="48">
@@ -2088,10 +2088,10 @@
       <c r="BL16" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM16" t="s" s="0">
+      <c r="BM16" t="s">
         <v>134</v>
       </c>
-      <c r="BN16" t="s" s="0">
+      <c r="BN16" t="s">
         <v>133</v>
       </c>
       <c r="BO16" s="48">
@@ -2261,20 +2261,20 @@
       <c r="AQ17" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR17" s="0">
+      <c r="AR17">
         <f>ROUND(AN17+AO17+AP17,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS17" t="s" s="0">
+      <c r="AS17" t="s">
         <v>107</v>
       </c>
       <c r="AT17" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU17" t="s" s="0">
+      <c r="AU17" t="s">
         <v>108</v>
       </c>
-      <c r="AV17" t="s" s="0">
+      <c r="AV17" t="s">
         <v>132</v>
       </c>
       <c r="AW17" s="48">
@@ -2480,20 +2480,20 @@
       <c r="AQ18" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR18" s="0">
+      <c r="AR18">
         <f>ROUND(AN18+AO18+AP18,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS18" t="s" s="0">
+      <c r="AS18" t="s">
         <v>107</v>
       </c>
       <c r="AT18" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU18" t="s" s="0">
+      <c r="AU18" t="s">
         <v>130</v>
       </c>
-      <c r="AV18" t="s" s="0">
+      <c r="AV18" t="s">
         <v>137</v>
       </c>
       <c r="AW18" s="48">
@@ -2532,10 +2532,10 @@
       <c r="BL18" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM18" t="s" s="0">
+      <c r="BM18" t="s">
         <v>153</v>
       </c>
-      <c r="BN18" t="s" s="0">
+      <c r="BN18" t="s">
         <v>152</v>
       </c>
       <c r="BO18" s="48">
@@ -2706,20 +2706,20 @@
       <c r="AQ20" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR20" t="e" s="0">
+      <c r="AR20" t="e">
         <f>ROUND(AN20+AO20+AP20,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS20" t="s" s="0">
+      <c r="AS20" t="s">
         <v>107</v>
       </c>
       <c r="AT20" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU20" t="s" s="0">
+      <c r="AU20" t="s">
         <v>155</v>
       </c>
-      <c r="AV20" t="s" s="0">
+      <c r="AV20" t="s">
         <v>156</v>
       </c>
       <c r="AW20" s="48">
@@ -2758,10 +2758,10 @@
       <c r="BL20" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM20" t="s" s="0">
+      <c r="BM20" t="s">
         <v>156</v>
       </c>
-      <c r="BN20" t="s" s="0">
+      <c r="BN20" t="s">
         <v>127</v>
       </c>
       <c r="BO20" s="48" t="e">
@@ -2931,20 +2931,20 @@
       <c r="AQ21" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR21" t="e" s="0">
+      <c r="AR21" t="e">
         <f t="shared" ref="AR21:AR23" si="30">ROUND(AN21+AO21+AP21,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS21" t="s" s="0">
+      <c r="AS21" t="s">
         <v>107</v>
       </c>
       <c r="AT21" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU21" t="s" s="0">
+      <c r="AU21" t="s">
         <v>131</v>
       </c>
-      <c r="AV21" t="s" s="0">
+      <c r="AV21" t="s">
         <v>157</v>
       </c>
       <c r="AW21" s="48">
@@ -2983,10 +2983,10 @@
       <c r="BL21" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM21" t="s" s="0">
+      <c r="BM21" t="s">
         <v>108</v>
       </c>
-      <c r="BN21" t="s" s="0">
+      <c r="BN21" t="s">
         <v>108</v>
       </c>
       <c r="BO21" s="48" t="e">
@@ -3156,20 +3156,20 @@
       <c r="AQ22" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR22" t="e" s="0">
+      <c r="AR22" t="e">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS22" t="s" s="0">
+      <c r="AS22" t="s">
         <v>107</v>
       </c>
       <c r="AT22" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU22" t="s" s="0">
+      <c r="AU22" t="s">
         <v>158</v>
       </c>
-      <c r="AV22" t="s" s="0">
+      <c r="AV22" t="s">
         <v>159</v>
       </c>
       <c r="AW22" s="48">
@@ -3208,10 +3208,10 @@
       <c r="BL22" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM22" t="s" s="0">
+      <c r="BM22" t="s">
         <v>108</v>
       </c>
-      <c r="BN22" t="s" s="0">
+      <c r="BN22" t="s">
         <v>108</v>
       </c>
       <c r="BO22" s="48" t="e">
@@ -3381,20 +3381,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" t="e" s="0">
+      <c r="AR23" t="e">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>160</v>
       </c>
       <c r="AW23" s="48">
@@ -3433,10 +3433,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48" t="e">
@@ -3493,14 +3493,14 @@
       <c r="F31" s="46">
         <v>2</v>
       </c>
-      <c r="G31" t="s" s="0">
+      <c r="G31" t="s">
         <v>128</v>
       </c>
       <c r="H31" s="46">
         <f>F31*G31</f>
         <v>600</v>
       </c>
-      <c r="I31" t="s" s="0">
+      <c r="I31" t="s">
         <v>127</v>
       </c>
       <c r="J31" s="46">
@@ -3628,20 +3628,20 @@
       <c r="AQ31" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR31" s="0">
+      <c r="AR31">
         <f>ROUND(AN31+AO31+AP31,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS31" t="s" s="0">
+      <c r="AS31" t="s">
         <v>107</v>
       </c>
       <c r="AT31" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU31" t="s" s="0">
+      <c r="AU31" t="s">
         <v>162</v>
       </c>
-      <c r="AV31" t="s" s="0">
+      <c r="AV31" t="s">
         <v>167</v>
       </c>
       <c r="AW31" s="48">
@@ -3680,10 +3680,10 @@
       <c r="BL31" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM31" t="s" s="0">
+      <c r="BM31" t="s">
         <v>108</v>
       </c>
-      <c r="BN31" t="s" s="0">
+      <c r="BN31" t="s">
         <v>108</v>
       </c>
       <c r="BO31" s="48">
@@ -3718,14 +3718,14 @@
       <c r="F32" s="46">
         <v>2</v>
       </c>
-      <c r="G32" t="s" s="0">
+      <c r="G32" t="s">
         <v>129</v>
       </c>
       <c r="H32" s="46">
         <f>F32*G32</f>
         <v>800</v>
       </c>
-      <c r="I32" t="s" s="0">
+      <c r="I32" t="s">
         <v>127</v>
       </c>
       <c r="J32" s="46">
@@ -3853,20 +3853,20 @@
       <c r="AQ32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR32" s="0">
+      <c r="AR32">
         <f>ROUND(AN32+AO32+AP32,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS32" t="s" s="0">
+      <c r="AS32" t="s">
         <v>107</v>
       </c>
       <c r="AT32" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU32" t="s" s="0">
+      <c r="AU32" t="s">
         <v>168</v>
       </c>
-      <c r="AV32" t="s" s="0">
+      <c r="AV32" t="s">
         <v>169</v>
       </c>
       <c r="AW32" s="48">
@@ -3905,10 +3905,10 @@
       <c r="BL32" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM32" t="s" s="0">
+      <c r="BM32" t="s">
         <v>108</v>
       </c>
-      <c r="BN32" t="s" s="0">
+      <c r="BN32" t="s">
         <v>108</v>
       </c>
       <c r="BO32" s="48">
@@ -3943,14 +3943,14 @@
       <c r="F33" s="46">
         <v>2</v>
       </c>
-      <c r="G33" t="s" s="0">
+      <c r="G33" t="s">
         <v>161</v>
       </c>
       <c r="H33" s="46">
         <f>F33*G33</f>
         <v>1000</v>
       </c>
-      <c r="I33" t="s" s="0">
+      <c r="I33" t="s">
         <v>127</v>
       </c>
       <c r="J33" s="46">
@@ -4078,20 +4078,20 @@
       <c r="AQ33" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR33" s="0">
+      <c r="AR33">
         <f>ROUND(AN33+AO33+AP33,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS33" t="s" s="0">
+      <c r="AS33" t="s">
         <v>107</v>
       </c>
       <c r="AT33" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU33" t="s" s="0">
+      <c r="AU33" t="s">
         <v>108</v>
       </c>
-      <c r="AV33" t="s" s="0">
+      <c r="AV33" t="s">
         <v>170</v>
       </c>
       <c r="AW33" s="48">
@@ -4130,10 +4130,10 @@
       <c r="BL33" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM33" t="s" s="0">
+      <c r="BM33" t="s">
         <v>108</v>
       </c>
-      <c r="BN33" t="s" s="0">
+      <c r="BN33" t="s">
         <v>108</v>
       </c>
       <c r="BO33" s="48">
@@ -4169,14 +4169,14 @@
       <c r="F35" s="46">
         <v>2</v>
       </c>
-      <c r="G35" t="s" s="0">
+      <c r="G35" t="s">
         <v>128</v>
       </c>
       <c r="H35" s="46">
         <f>F35*G35</f>
         <v>600</v>
       </c>
-      <c r="I35" t="s" s="0">
+      <c r="I35" t="s">
         <v>127</v>
       </c>
       <c r="J35" s="46">
@@ -4304,20 +4304,20 @@
       <c r="AQ35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR35" s="0">
+      <c r="AR35">
         <f>ROUND(AN35+AO35+AP35,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS35" t="s" s="0">
+      <c r="AS35" t="s">
         <v>107</v>
       </c>
       <c r="AT35" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU35" t="s" s="0">
+      <c r="AU35" t="s">
         <v>171</v>
       </c>
-      <c r="AV35" t="s" s="0">
+      <c r="AV35" t="s">
         <v>172</v>
       </c>
       <c r="AW35" s="48">
@@ -4356,10 +4356,10 @@
       <c r="BL35" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM35" t="s" s="0">
+      <c r="BM35" t="s">
         <v>108</v>
       </c>
-      <c r="BN35" t="s" s="0">
+      <c r="BN35" t="s">
         <v>108</v>
       </c>
       <c r="BO35" s="48">
@@ -4394,14 +4394,14 @@
       <c r="F36" s="46">
         <v>2</v>
       </c>
-      <c r="G36" t="s" s="0">
+      <c r="G36" t="s">
         <v>129</v>
       </c>
       <c r="H36" s="46">
         <f>F36*G36</f>
         <v>800</v>
       </c>
-      <c r="I36" t="s" s="0">
+      <c r="I36" t="s">
         <v>127</v>
       </c>
       <c r="J36" s="46">
@@ -4529,20 +4529,20 @@
       <c r="AQ36" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR36" s="0">
+      <c r="AR36">
         <f>ROUND(AN36+AO36+AP36,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS36" t="s" s="0">
+      <c r="AS36" t="s">
         <v>107</v>
       </c>
       <c r="AT36" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU36" t="s" s="0">
+      <c r="AU36" t="s">
         <v>173</v>
       </c>
-      <c r="AV36" t="s" s="0">
+      <c r="AV36" t="s">
         <v>174</v>
       </c>
       <c r="AW36" s="48">
@@ -4581,10 +4581,10 @@
       <c r="BL36" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM36" t="s" s="0">
+      <c r="BM36" t="s">
         <v>108</v>
       </c>
-      <c r="BN36" t="s" s="0">
+      <c r="BN36" t="s">
         <v>108</v>
       </c>
       <c r="BO36" s="48">
@@ -4619,14 +4619,14 @@
       <c r="F37" s="46">
         <v>2</v>
       </c>
-      <c r="G37" t="s" s="0">
+      <c r="G37" t="s">
         <v>161</v>
       </c>
       <c r="H37" s="46">
         <f>F37*G37</f>
         <v>1000</v>
       </c>
-      <c r="I37" t="s" s="0">
+      <c r="I37" t="s">
         <v>127</v>
       </c>
       <c r="J37" s="46">
@@ -4754,20 +4754,20 @@
       <c r="AQ37" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR37" s="0">
+      <c r="AR37">
         <f>ROUND(AN37+AO37+AP37,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS37" t="s" s="0">
+      <c r="AS37" t="s">
         <v>107</v>
       </c>
       <c r="AT37" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU37" t="s" s="0">
+      <c r="AU37" t="s">
         <v>108</v>
       </c>
-      <c r="AV37" t="s" s="0">
+      <c r="AV37" t="s">
         <v>170</v>
       </c>
       <c r="AW37" s="48">
@@ -4806,10 +4806,10 @@
       <c r="BL37" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM37" t="s" s="0">
+      <c r="BM37" t="s">
         <v>108</v>
       </c>
-      <c r="BN37" t="s" s="0">
+      <c r="BN37" t="s">
         <v>108</v>
       </c>
       <c r="BO37" s="48">
@@ -4835,34 +4835,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -6388,14 +6388,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -6523,20 +6523,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -6575,10 +6575,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -6753,32 +6753,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -8304,14 +8304,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -8439,12 +8439,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -8654,34 +8654,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -10207,14 +10207,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -10342,20 +10342,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -10394,10 +10394,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -10572,32 +10572,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -12123,14 +12123,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -12258,12 +12258,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -12473,34 +12473,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -14026,14 +14026,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -14161,20 +14161,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -14213,10 +14213,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -14391,32 +14391,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -15942,14 +15942,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -16077,12 +16077,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -16292,34 +16292,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -17980,20 +17980,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>175</v>
       </c>
       <c r="AW23" s="48">
@@ -18032,10 +18032,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>175</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>176</v>
       </c>
       <c r="BO23" s="48">
@@ -18207,34 +18207,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -19895,20 +19895,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>131</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -19947,10 +19947,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>150</v>
       </c>
       <c r="BO23" s="48">
@@ -20122,32 +20122,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -21673,14 +21673,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -21808,12 +21808,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -22023,34 +22023,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -23576,14 +23576,14 @@
       <c r="F23" s="46">
         <v>50</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>1000</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -23711,20 +23711,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>57.048000000000002</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>181</v>
       </c>
       <c r="AW23" s="48">
@@ -23763,10 +23763,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>183</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>182</v>
       </c>
       <c r="BO23" s="48">
@@ -23938,34 +23938,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -25626,20 +25626,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -25678,10 +25678,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>155</v>
       </c>
       <c r="BO23" s="48">
@@ -25854,34 +25854,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -27407,14 +27407,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>60</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -27542,20 +27542,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>55.89</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>177</v>
       </c>
       <c r="AW23" s="48">
@@ -27594,10 +27594,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>177</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>130</v>
       </c>
       <c r="BO23" s="48">
@@ -27769,32 +27769,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -29320,14 +29320,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -29455,12 +29455,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -29670,34 +29670,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -31223,14 +31223,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>60</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -31358,20 +31358,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>55.89</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>178</v>
       </c>
       <c r="AW23" s="48">
@@ -31410,10 +31410,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>178</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>150</v>
       </c>
       <c r="BO23" s="48">
@@ -31588,34 +31588,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -33141,14 +33141,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>60</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -33276,20 +33276,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>56.46</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>178</v>
       </c>
       <c r="AW23" s="48">
@@ -33328,10 +33328,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>178</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>158</v>
       </c>
       <c r="BO23" s="48">
@@ -33506,32 +33506,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -35057,14 +35057,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -35192,12 +35192,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -35407,32 +35407,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -37093,20 +37093,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -37145,10 +37145,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>164</v>
       </c>
       <c r="BO23" s="48">
@@ -37323,32 +37323,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -39009,12 +39009,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -39224,34 +39224,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -40777,14 +40777,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -40912,20 +40912,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>195</v>
       </c>
       <c r="AW23" s="48">
@@ -40964,10 +40964,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48">
@@ -41140,32 +41140,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -42691,14 +42691,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -42826,12 +42826,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -43041,34 +43041,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -44594,14 +44594,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -44729,20 +44729,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>158</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>179</v>
       </c>
       <c r="AW23" s="48">
@@ -44781,10 +44781,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>180</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>131</v>
       </c>
       <c r="BO23" s="48">
@@ -44960,32 +44960,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -46511,14 +46511,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -46646,12 +46646,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -46862,34 +46862,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -48415,14 +48415,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -48550,20 +48550,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
-        <v>107</v>
+      <c r="AS23" t="s">
+        <v>194</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>132</v>
       </c>
       <c r="AW23" s="48">
@@ -48602,10 +48602,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48">

</xml_diff>

<commit_message>
Fixes For The Failed Test Scenarios Of SOM And POM Modules
Fixes For The Failed Test Scenarios Of SOM And POM Modules
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4118" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4118" uniqueCount="195">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -602,9 +602,6 @@
   </si>
   <si>
     <t>56.96721</t>
-  </si>
-  <si>
-    <t>TVS-RM-KDK-101</t>
   </si>
   <si>
     <t>ROAU-RM-KDK-01</t>
@@ -6528,7 +6525,7 @@
         <v>186.32</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -8290,10 +8287,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -8444,7 +8441,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -10193,10 +10190,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -10347,7 +10344,7 @@
         <v>186.32</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -12109,10 +12106,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -12263,7 +12260,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -14012,10 +14009,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -14166,7 +14163,7 @@
         <v>186.32</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -15928,10 +15925,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -16082,7 +16079,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -17831,10 +17828,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -17985,7 +17982,7 @@
         <v>846.99</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -19746,10 +19743,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -19900,7 +19897,7 @@
         <v>282.33</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -21659,10 +21656,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -21813,7 +21810,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -23562,10 +23559,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -23716,7 +23713,7 @@
         <v>57.048000000000002</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -25477,10 +25474,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -25631,7 +25628,7 @@
         <v>282.33</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -27393,10 +27390,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -27547,7 +27544,7 @@
         <v>55.89</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -29306,10 +29303,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>117</v>
+        <v>185</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>117</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -29460,7 +29457,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -31209,10 +31206,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -31363,7 +31360,7 @@
         <v>55.89</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -33127,10 +33124,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -33281,7 +33278,7 @@
         <v>56.46</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -35043,10 +35040,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>117</v>
+        <v>185</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>117</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -35197,7 +35194,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -36944,10 +36941,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -37098,7 +37095,7 @@
         <v>282.33</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -38860,10 +38857,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -39014,7 +39011,7 @@
         <v>282.33</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -40763,10 +40760,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -40917,7 +40914,7 @@
         <v>282.33</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -40926,7 +40923,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -42677,10 +42674,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -42831,7 +42828,7 @@
         <v>282.33</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -44580,10 +44577,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -44734,7 +44731,7 @@
         <v>186.32</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -46497,10 +46494,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -46651,7 +46648,7 @@
         <v>18.824999999999999</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -48401,10 +48398,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -48555,7 +48552,7 @@
         <v>186.32</v>
       </c>
       <c r="AS23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>

</xml_diff>

<commit_message>
Fixes For The failed Test Scenarios Of SOM, POM And HRM Modules
Fixes For The failed Test Scenarios Of SOM, POM And HRM Modules
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="18" activeTab="18"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="19" activeTab="19"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4113" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4154" uniqueCount="205">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -583,12 +583,6 @@
     <t>1.334</t>
   </si>
   <si>
-    <t>55.89</t>
-  </si>
-  <si>
-    <t>56.46</t>
-  </si>
-  <si>
     <t>185.02695</t>
   </si>
   <si>
@@ -638,6 +632,39 @@
   </si>
   <si>
     <t>ROAU-KDK-DIS-SERVICE-01</t>
+  </si>
+  <si>
+    <t>558.96</t>
+  </si>
+  <si>
+    <t>8.671</t>
+  </si>
+  <si>
+    <t>9.338</t>
+  </si>
+  <si>
+    <t>566.36571</t>
+  </si>
+  <si>
+    <t>10.005</t>
+  </si>
+  <si>
+    <t>565.872</t>
+  </si>
+  <si>
+    <t>570.48</t>
+  </si>
+  <si>
+    <t>11.339</t>
+  </si>
+  <si>
+    <t>565.73647</t>
+  </si>
+  <si>
+    <t>12.006</t>
+  </si>
+  <si>
+    <t>566</t>
   </si>
 </sst>
 </file>
@@ -1424,7 +1451,7 @@
   <dimension ref="A8:BR37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="27.28515625"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:70" ht="15.75" thickBot="1"/>
@@ -1592,10 +1619,10 @@
       <c r="AT9" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU9" t="s">
+      <c r="AU9" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV9" t="s">
+      <c r="AV9" t="s" s="0">
         <v>143</v>
       </c>
       <c r="AW9" s="48">
@@ -1636,10 +1663,10 @@
       <c r="BL9" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM9" t="s">
+      <c r="BM9" t="s" s="0">
         <v>146</v>
       </c>
-      <c r="BN9" t="s">
+      <c r="BN9" t="s" s="0">
         <v>147</v>
       </c>
       <c r="BO9" s="48" t="e">
@@ -1811,20 +1838,20 @@
       <c r="AQ15" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR15" t="e">
+      <c r="AR15" t="e" s="0">
         <f>ROUND(AN15+AO15+AP15,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS15" t="s">
+      <c r="AS15" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT15" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU15" t="s">
+      <c r="AU15" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="AV15" t="s">
+      <c r="AV15" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW15" s="48">
@@ -1863,10 +1890,10 @@
       <c r="BL15" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM15" t="s">
+      <c r="BM15" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN15" t="s">
+      <c r="BN15" t="s" s="0">
         <v>150</v>
       </c>
       <c r="BO15" s="48" t="e">
@@ -2036,20 +2063,20 @@
       <c r="AQ16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR16">
+      <c r="AR16" s="0">
         <f>ROUND(AN16+AO16+AP16,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS16" t="s">
+      <c r="AS16" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT16" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU16" t="s">
+      <c r="AU16" t="s" s="0">
         <v>135</v>
       </c>
-      <c r="AV16" t="s">
+      <c r="AV16" t="s" s="0">
         <v>136</v>
       </c>
       <c r="AW16" s="48">
@@ -2088,10 +2115,10 @@
       <c r="BL16" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM16" t="s">
+      <c r="BM16" t="s" s="0">
         <v>134</v>
       </c>
-      <c r="BN16" t="s">
+      <c r="BN16" t="s" s="0">
         <v>133</v>
       </c>
       <c r="BO16" s="48">
@@ -2261,20 +2288,20 @@
       <c r="AQ17" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR17">
+      <c r="AR17" s="0">
         <f>ROUND(AN17+AO17+AP17,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS17" t="s">
+      <c r="AS17" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT17" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU17" t="s">
+      <c r="AU17" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV17" t="s">
+      <c r="AV17" t="s" s="0">
         <v>132</v>
       </c>
       <c r="AW17" s="48">
@@ -2480,20 +2507,20 @@
       <c r="AQ18" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR18">
+      <c r="AR18" s="0">
         <f>ROUND(AN18+AO18+AP18,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS18" t="s">
+      <c r="AS18" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT18" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU18" t="s">
+      <c r="AU18" t="s" s="0">
         <v>130</v>
       </c>
-      <c r="AV18" t="s">
+      <c r="AV18" t="s" s="0">
         <v>137</v>
       </c>
       <c r="AW18" s="48">
@@ -2532,10 +2559,10 @@
       <c r="BL18" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM18" t="s">
+      <c r="BM18" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="BN18" t="s">
+      <c r="BN18" t="s" s="0">
         <v>152</v>
       </c>
       <c r="BO18" s="48">
@@ -2706,20 +2733,20 @@
       <c r="AQ20" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR20" t="e">
+      <c r="AR20" t="e" s="0">
         <f>ROUND(AN20+AO20+AP20,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS20" t="s">
+      <c r="AS20" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT20" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU20" t="s">
+      <c r="AU20" t="s" s="0">
         <v>155</v>
       </c>
-      <c r="AV20" t="s">
+      <c r="AV20" t="s" s="0">
         <v>156</v>
       </c>
       <c r="AW20" s="48">
@@ -2758,10 +2785,10 @@
       <c r="BL20" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM20" t="s">
+      <c r="BM20" t="s" s="0">
         <v>156</v>
       </c>
-      <c r="BN20" t="s">
+      <c r="BN20" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO20" s="48" t="e">
@@ -2931,20 +2958,20 @@
       <c r="AQ21" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR21" t="e">
+      <c r="AR21" t="e" s="0">
         <f t="shared" ref="AR21:AR23" si="30">ROUND(AN21+AO21+AP21,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS21" t="s">
+      <c r="AS21" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT21" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU21" t="s">
+      <c r="AU21" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="AV21" t="s">
+      <c r="AV21" t="s" s="0">
         <v>157</v>
       </c>
       <c r="AW21" s="48">
@@ -2983,10 +3010,10 @@
       <c r="BL21" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM21" t="s">
+      <c r="BM21" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN21" t="s">
+      <c r="BN21" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO21" s="48" t="e">
@@ -3156,20 +3183,20 @@
       <c r="AQ22" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR22" t="e">
+      <c r="AR22" t="e" s="0">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS22" t="s">
+      <c r="AS22" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT22" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU22" t="s">
+      <c r="AU22" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="AV22" t="s">
+      <c r="AV22" t="s" s="0">
         <v>159</v>
       </c>
       <c r="AW22" s="48">
@@ -3208,10 +3235,10 @@
       <c r="BL22" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM22" t="s">
+      <c r="BM22" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN22" t="s">
+      <c r="BN22" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO22" s="48" t="e">
@@ -3381,20 +3408,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" t="e">
+      <c r="AR23" t="e" s="0">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>160</v>
       </c>
       <c r="AW23" s="48">
@@ -3433,10 +3460,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO23" s="48" t="e">
@@ -3493,14 +3520,14 @@
       <c r="F31" s="46">
         <v>2</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" t="s" s="0">
         <v>128</v>
       </c>
       <c r="H31" s="46">
         <f>F31*G31</f>
         <v>600</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J31" s="46">
@@ -3628,20 +3655,20 @@
       <c r="AQ31" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR31">
+      <c r="AR31" s="0">
         <f>ROUND(AN31+AO31+AP31,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS31" t="s">
+      <c r="AS31" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT31" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU31" t="s">
+      <c r="AU31" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="AV31" t="s">
+      <c r="AV31" t="s" s="0">
         <v>167</v>
       </c>
       <c r="AW31" s="48">
@@ -3680,10 +3707,10 @@
       <c r="BL31" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM31" t="s">
+      <c r="BM31" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN31" t="s">
+      <c r="BN31" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO31" s="48">
@@ -3718,14 +3745,14 @@
       <c r="F32" s="46">
         <v>2</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" t="s" s="0">
         <v>129</v>
       </c>
       <c r="H32" s="46">
         <f>F32*G32</f>
         <v>800</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J32" s="46">
@@ -3853,20 +3880,20 @@
       <c r="AQ32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR32">
+      <c r="AR32" s="0">
         <f>ROUND(AN32+AO32+AP32,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS32" t="s">
+      <c r="AS32" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT32" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU32" t="s">
+      <c r="AU32" t="s" s="0">
         <v>168</v>
       </c>
-      <c r="AV32" t="s">
+      <c r="AV32" t="s" s="0">
         <v>169</v>
       </c>
       <c r="AW32" s="48">
@@ -3905,10 +3932,10 @@
       <c r="BL32" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM32" t="s">
+      <c r="BM32" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN32" t="s">
+      <c r="BN32" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO32" s="48">
@@ -3943,14 +3970,14 @@
       <c r="F33" s="46">
         <v>2</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" t="s" s="0">
         <v>161</v>
       </c>
       <c r="H33" s="46">
         <f>F33*G33</f>
         <v>1000</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J33" s="46">
@@ -4078,20 +4105,20 @@
       <c r="AQ33" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR33">
+      <c r="AR33" s="0">
         <f>ROUND(AN33+AO33+AP33,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS33" t="s">
+      <c r="AS33" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT33" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU33" t="s">
+      <c r="AU33" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV33" t="s">
+      <c r="AV33" t="s" s="0">
         <v>170</v>
       </c>
       <c r="AW33" s="48">
@@ -4130,10 +4157,10 @@
       <c r="BL33" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM33" t="s">
+      <c r="BM33" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN33" t="s">
+      <c r="BN33" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO33" s="48">
@@ -4169,14 +4196,14 @@
       <c r="F35" s="46">
         <v>2</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" t="s" s="0">
         <v>128</v>
       </c>
       <c r="H35" s="46">
         <f>F35*G35</f>
         <v>600</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J35" s="46">
@@ -4304,20 +4331,20 @@
       <c r="AQ35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR35">
+      <c r="AR35" s="0">
         <f>ROUND(AN35+AO35+AP35,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS35" t="s">
+      <c r="AS35" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT35" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU35" t="s">
+      <c r="AU35" t="s" s="0">
         <v>171</v>
       </c>
-      <c r="AV35" t="s">
+      <c r="AV35" t="s" s="0">
         <v>172</v>
       </c>
       <c r="AW35" s="48">
@@ -4356,10 +4383,10 @@
       <c r="BL35" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM35" t="s">
+      <c r="BM35" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN35" t="s">
+      <c r="BN35" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO35" s="48">
@@ -4394,14 +4421,14 @@
       <c r="F36" s="46">
         <v>2</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36" t="s" s="0">
         <v>129</v>
       </c>
       <c r="H36" s="46">
         <f>F36*G36</f>
         <v>800</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J36" s="46">
@@ -4529,20 +4556,20 @@
       <c r="AQ36" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR36">
+      <c r="AR36" s="0">
         <f>ROUND(AN36+AO36+AP36,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS36" t="s">
+      <c r="AS36" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT36" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU36" t="s">
+      <c r="AU36" t="s" s="0">
         <v>173</v>
       </c>
-      <c r="AV36" t="s">
+      <c r="AV36" t="s" s="0">
         <v>174</v>
       </c>
       <c r="AW36" s="48">
@@ -4581,10 +4608,10 @@
       <c r="BL36" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM36" t="s">
+      <c r="BM36" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN36" t="s">
+      <c r="BN36" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO36" s="48">
@@ -4619,14 +4646,14 @@
       <c r="F37" s="46">
         <v>2</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" t="s" s="0">
         <v>161</v>
       </c>
       <c r="H37" s="46">
         <f>F37*G37</f>
         <v>1000</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J37" s="46">
@@ -4754,20 +4781,20 @@
       <c r="AQ37" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR37">
+      <c r="AR37" s="0">
         <f>ROUND(AN37+AO37+AP37,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS37" t="s">
+      <c r="AS37" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT37" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU37" t="s">
+      <c r="AU37" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV37" t="s">
+      <c r="AV37" t="s" s="0">
         <v>170</v>
       </c>
       <c r="AW37" s="48">
@@ -4806,10 +4833,10 @@
       <c r="BL37" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM37" t="s">
+      <c r="BM37" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN37" t="s">
+      <c r="BN37" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO37" s="48">
@@ -4835,34 +4862,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -6374,10 +6401,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -6388,14 +6415,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -6523,20 +6550,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>164</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -6575,10 +6602,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>163</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -6753,32 +6780,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -8290,10 +8317,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -8304,14 +8331,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -8439,12 +8466,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -8654,34 +8681,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -10193,10 +10220,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -10207,14 +10234,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -10342,20 +10369,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>164</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -10394,10 +10421,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>163</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -10572,32 +10599,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -12109,10 +12136,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -12123,14 +12150,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -12258,12 +12285,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -12473,34 +12500,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -14012,10 +14039,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -14026,14 +14053,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -14161,20 +14188,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>164</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -14213,10 +14240,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>163</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -14391,32 +14418,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -15928,10 +15955,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -15942,14 +15969,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -16077,12 +16104,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -16292,34 +16319,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -17831,10 +17858,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -17980,20 +18007,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>175</v>
       </c>
       <c r="AW23" s="48">
@@ -18032,10 +18059,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>175</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>176</v>
       </c>
       <c r="BO23" s="48">
@@ -18043,8 +18070,8 @@
         <v>846.99</v>
       </c>
       <c r="BP23" s="61">
-        <f>BN23+AW23</f>
-        <v>0.66666666666666663</v>
+        <f>ROUND((BN23+AW23),3)</f>
+        <v>2.0009999999999999</v>
       </c>
       <c r="BQ23" s="50">
         <v>88363222</v>
@@ -18207,34 +18234,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -19746,10 +19773,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -19895,20 +19922,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -19947,10 +19974,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>150</v>
       </c>
       <c r="BO23" s="48">
@@ -19958,7 +19985,7 @@
         <v>282.33</v>
       </c>
       <c r="BP23" s="4">
-        <f>BN23+AW23</f>
+        <f>ROUND((BN23+AW23),3)</f>
         <v>8</v>
       </c>
       <c r="BQ23" s="50">
@@ -20122,32 +20149,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -21659,10 +21686,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -21673,14 +21700,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -21808,12 +21835,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -22023,34 +22050,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -23562,10 +23589,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -23576,14 +23603,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23">
-        <v>200</v>
+      <c r="G23" t="s" s="0">
+        <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -23711,21 +23738,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>570.48</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
-        <v>181</v>
+      <c r="AV23" t="s" s="0">
+        <v>200</v>
       </c>
       <c r="AW23" s="16">
         <f>AM23</f>
@@ -23763,11 +23790,11 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>183</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>182</v>
+      <c r="BM23" t="s" s="0">
+        <v>204</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>203</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),3)</f>
@@ -23938,34 +23965,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -25477,10 +25504,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -25626,20 +25653,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -25678,10 +25705,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>155</v>
       </c>
       <c r="BO23" s="48">
@@ -25854,34 +25881,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -27393,10 +27420,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -27407,14 +27434,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23">
-        <v>200</v>
+      <c r="G23" t="s" s="0">
+        <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -27542,21 +27569,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>558.96</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
-        <v>177</v>
+      <c r="AV23" t="s" s="0">
+        <v>194</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -27594,19 +27621,19 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>177</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>130</v>
+      <c r="BM23" t="s" s="0">
+        <v>199</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>198</v>
       </c>
       <c r="BO23" s="48">
-        <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>127.75714000000001</v>
+        <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),3)</f>
+        <v>566.36599999999999</v>
       </c>
       <c r="BP23" s="4">
-        <f>BN23+AW23</f>
-        <v>4.666666666666667</v>
+        <f>ROUND((BN23+AW23),3)</f>
+        <v>9.3379999999999992</v>
       </c>
       <c r="BQ23" s="50">
         <v>88363222</v>
@@ -27769,32 +27796,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -29306,10 +29333,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -29320,14 +29347,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>200</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -29455,12 +29482,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>188.22</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -29506,7 +29533,7 @@
         <v>188.22</v>
       </c>
       <c r="BP23" s="4">
-        <f>BN23+AW23</f>
+        <f>ROUND((BN23+AW23),3)</f>
         <v>2</v>
       </c>
       <c r="BQ23" s="50">
@@ -29670,34 +29697,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -31209,10 +31236,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -31223,15 +31250,15 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23">
-        <v>200</v>
+      <c r="G23" t="s" s="0">
+        <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
-        <v>115</v>
+      <c r="I23" t="s" s="0">
+        <v>127</v>
       </c>
       <c r="J23" s="46">
         <v>2</v>
@@ -31358,21 +31385,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>564.66</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
-        <v>178</v>
+      <c r="AV23" t="s" s="0">
+        <v>194</v>
       </c>
       <c r="AW23" s="16">
         <f>AM23</f>
@@ -31410,19 +31437,19 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>178</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>150</v>
+      <c r="BM23" t="s" s="0">
+        <v>194</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>196</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>107.28</v>
       </c>
-      <c r="BP23" s="4">
-        <f>BN23+AW23</f>
-        <v>6.666666666666667</v>
+      <c r="BP23" s="61">
+        <f>ROUND((BN23+AW23),3)</f>
+        <v>6.6669999999999998</v>
       </c>
       <c r="BQ23" s="50">
         <v>88363222</v>
@@ -31588,34 +31615,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -33127,10 +33154,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -33141,15 +33168,15 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23">
-        <v>200</v>
+      <c r="G23" t="s" s="0">
+        <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
-        <v>115</v>
+      <c r="I23" t="s" s="0">
+        <v>127</v>
       </c>
       <c r="J23" s="46">
         <v>2</v>
@@ -33276,21 +33303,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>564.66</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
-        <v>178</v>
+      <c r="AV23" t="s" s="0">
+        <v>194</v>
       </c>
       <c r="AW23" s="16">
         <f>AM23</f>
@@ -33328,19 +33355,19 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>178</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>158</v>
+      <c r="BM23" t="s" s="0">
+        <v>194</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>195</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
         <v>76.787999999999997</v>
       </c>
-      <c r="BP23" s="4">
-        <f>BN23+AW23</f>
-        <v>16.666666666666668</v>
+      <c r="BP23" s="61">
+        <f>ROUND((BN23+AW23),3)</f>
+        <v>8.6709999999999994</v>
       </c>
       <c r="BQ23" s="50">
         <v>88363222</v>
@@ -33506,32 +33533,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -35043,10 +35070,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -35057,14 +35084,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -35192,12 +35219,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -35407,32 +35434,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -36944,10 +36971,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -37093,20 +37120,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -37145,10 +37172,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>164</v>
       </c>
       <c r="BO23" s="48">
@@ -37323,32 +37350,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -38860,10 +38887,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -39009,12 +39036,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -39224,34 +39251,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -40763,10 +40790,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -40777,14 +40804,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -40912,21 +40939,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
-        <v>194</v>
+      <c r="AV23" t="s" s="0">
+        <v>192</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -40964,10 +40991,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO23" s="48">
@@ -41140,32 +41167,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -42677,10 +42704,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -42691,14 +42718,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -42826,12 +42853,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -43041,34 +43068,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -44580,10 +44607,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -44594,14 +44621,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -44729,21 +44756,21 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="AV23" t="s">
-        <v>179</v>
+      <c r="AV23" t="s" s="0">
+        <v>177</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -44781,10 +44808,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>180</v>
-      </c>
-      <c r="BN23" t="s">
+      <c r="BM23" t="s" s="0">
+        <v>178</v>
+      </c>
+      <c r="BN23" t="s" s="0">
         <v>131</v>
       </c>
       <c r="BO23" s="48">
@@ -44960,32 +44987,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -46497,10 +46524,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C23" s="45" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -46511,14 +46538,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -46646,12 +46673,12 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
@@ -46862,34 +46889,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -48401,10 +48428,10 @@
         <v>1</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="D23" s="45" t="s">
         <v>12</v>
@@ -48415,14 +48442,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -48550,20 +48577,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
-        <v>193</v>
+      <c r="AS23" t="s" s="0">
+        <v>191</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>132</v>
       </c>
       <c r="AW23" s="48">
@@ -48602,10 +48629,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO23" s="48">

</xml_diff>

<commit_message>
Subcontract Function And Subcontract Test Changes Fixes
Subcontract Function And Subcontract Test Changes Fixes
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="16" activeTab="16"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -21799,15 +21799,15 @@
         <v>0</v>
       </c>
       <c r="AL23" s="46">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AM23" s="46">
         <f>F23/AL23</f>
-        <v>2</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="AN23" s="46">
         <f>AI23/AM23</f>
-        <v>282.33</v>
+        <v>846.99</v>
       </c>
       <c r="AO23" s="46">
         <f>AJ23/AM23</f>
@@ -21822,7 +21822,7 @@
       </c>
       <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
-        <v>282.33</v>
+        <v>846.99</v>
       </c>
       <c r="AS23" t="s">
         <v>188</v>
@@ -21838,19 +21838,19 @@
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
-        <v>2</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="AX23" s="48">
         <f>AR23</f>
-        <v>282.33</v>
+        <v>846.99</v>
       </c>
       <c r="AY23" s="48">
         <f>AU23+AW23</f>
-        <v>14</v>
+        <v>12.666666666666666</v>
       </c>
       <c r="AZ23" s="48">
         <f>ROUND(((AU23*AV23)+(AW23*AX23))/(AU23+AW23),5)</f>
-        <v>282.33</v>
+        <v>312.04894999999999</v>
       </c>
       <c r="BA23" s="3"/>
       <c r="BB23" s="3" t="s">
@@ -21880,11 +21880,11 @@
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
-        <v>282.33</v>
+        <v>285.30189999999999</v>
       </c>
       <c r="BP23" s="4">
         <f>ROUND((BN23+AW23),3)</f>
-        <v>8</v>
+        <v>6.6669999999999998</v>
       </c>
       <c r="BQ23" s="50">
         <v>88363222</v>

</xml_diff>

<commit_message>
Fixes For The Cash Payment And Cash Receipt Scenarios
Fixes For The Cash Payment And Cash Receipt Scenarios
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5512" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5528" uniqueCount="230">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -727,6 +727,27 @@
   </si>
   <si>
     <t>294</t>
+  </si>
+  <si>
+    <t>1102</t>
+  </si>
+  <si>
+    <t>880.96853</t>
+  </si>
+  <si>
+    <t>1104</t>
+  </si>
+  <si>
+    <t>879.88404</t>
+  </si>
+  <si>
+    <t>1106</t>
+  </si>
+  <si>
+    <t>878.80347</t>
+  </si>
+  <si>
+    <t>1810.39779</t>
   </si>
 </sst>
 </file>
@@ -1574,7 +1595,7 @@
   <dimension ref="A8:BR37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="27.28515625"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:70" ht="15.75" thickBot="1"/>
@@ -1742,10 +1763,10 @@
       <c r="AT9" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU9" t="s">
+      <c r="AU9" t="s" s="0">
         <v>127</v>
       </c>
-      <c r="AV9" t="s">
+      <c r="AV9" t="s" s="0">
         <v>143</v>
       </c>
       <c r="AW9" s="48">
@@ -1786,10 +1807,10 @@
       <c r="BL9" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM9" t="s">
+      <c r="BM9" t="s" s="0">
         <v>146</v>
       </c>
-      <c r="BN9" t="s">
+      <c r="BN9" t="s" s="0">
         <v>147</v>
       </c>
       <c r="BO9" s="48" t="e">
@@ -1961,20 +1982,20 @@
       <c r="AQ15" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR15" t="e">
+      <c r="AR15" t="e" s="0">
         <f>ROUND(AN15+AO15+AP15,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS15" t="s">
+      <c r="AS15" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT15" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU15" t="s">
+      <c r="AU15" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="AV15" t="s">
+      <c r="AV15" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW15" s="48">
@@ -2013,10 +2034,10 @@
       <c r="BL15" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM15" t="s">
+      <c r="BM15" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN15" t="s">
+      <c r="BN15" t="s" s="0">
         <v>150</v>
       </c>
       <c r="BO15" s="48" t="e">
@@ -2186,20 +2207,20 @@
       <c r="AQ16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR16">
+      <c r="AR16" s="0">
         <f>ROUND(AN16+AO16+AP16,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS16" t="s">
+      <c r="AS16" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT16" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU16" t="s">
+      <c r="AU16" t="s" s="0">
         <v>135</v>
       </c>
-      <c r="AV16" t="s">
+      <c r="AV16" t="s" s="0">
         <v>136</v>
       </c>
       <c r="AW16" s="48">
@@ -2238,10 +2259,10 @@
       <c r="BL16" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM16" t="s">
+      <c r="BM16" t="s" s="0">
         <v>134</v>
       </c>
-      <c r="BN16" t="s">
+      <c r="BN16" t="s" s="0">
         <v>133</v>
       </c>
       <c r="BO16" s="48">
@@ -2411,20 +2432,20 @@
       <c r="AQ17" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR17">
+      <c r="AR17" s="0">
         <f>ROUND(AN17+AO17+AP17,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS17" t="s">
+      <c r="AS17" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT17" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU17" t="s">
+      <c r="AU17" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV17" t="s">
+      <c r="AV17" t="s" s="0">
         <v>132</v>
       </c>
       <c r="AW17" s="48">
@@ -2630,20 +2651,20 @@
       <c r="AQ18" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR18">
+      <c r="AR18" s="0">
         <f>ROUND(AN18+AO18+AP18,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS18" t="s">
+      <c r="AS18" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT18" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU18" t="s">
+      <c r="AU18" t="s" s="0">
         <v>130</v>
       </c>
-      <c r="AV18" t="s">
+      <c r="AV18" t="s" s="0">
         <v>137</v>
       </c>
       <c r="AW18" s="48">
@@ -2682,10 +2703,10 @@
       <c r="BL18" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM18" t="s">
+      <c r="BM18" t="s" s="0">
         <v>153</v>
       </c>
-      <c r="BN18" t="s">
+      <c r="BN18" t="s" s="0">
         <v>152</v>
       </c>
       <c r="BO18" s="48">
@@ -2856,20 +2877,20 @@
       <c r="AQ20" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR20" t="e">
+      <c r="AR20" t="e" s="0">
         <f>ROUND(AN20+AO20+AP20,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS20" t="s">
+      <c r="AS20" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT20" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU20" t="s">
+      <c r="AU20" t="s" s="0">
         <v>155</v>
       </c>
-      <c r="AV20" t="s">
+      <c r="AV20" t="s" s="0">
         <v>156</v>
       </c>
       <c r="AW20" s="48">
@@ -2908,10 +2929,10 @@
       <c r="BL20" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM20" t="s">
+      <c r="BM20" t="s" s="0">
         <v>156</v>
       </c>
-      <c r="BN20" t="s">
+      <c r="BN20" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO20" s="48" t="e">
@@ -3081,20 +3102,20 @@
       <c r="AQ21" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR21" t="e">
+      <c r="AR21" t="e" s="0">
         <f t="shared" ref="AR21:AR23" si="30">ROUND(AN21+AO21+AP21,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS21" t="s">
+      <c r="AS21" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT21" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU21" t="s">
+      <c r="AU21" t="s" s="0">
         <v>131</v>
       </c>
-      <c r="AV21" t="s">
+      <c r="AV21" t="s" s="0">
         <v>157</v>
       </c>
       <c r="AW21" s="48">
@@ -3133,10 +3154,10 @@
       <c r="BL21" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM21" t="s">
+      <c r="BM21" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN21" t="s">
+      <c r="BN21" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO21" s="48" t="e">
@@ -3306,20 +3327,20 @@
       <c r="AQ22" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR22" t="e">
+      <c r="AR22" t="e" s="0">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS22" t="s">
+      <c r="AS22" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT22" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU22" t="s">
+      <c r="AU22" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="AV22" t="s">
+      <c r="AV22" t="s" s="0">
         <v>159</v>
       </c>
       <c r="AW22" s="48">
@@ -3358,10 +3379,10 @@
       <c r="BL22" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM22" t="s">
+      <c r="BM22" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN22" t="s">
+      <c r="BN22" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO22" s="48" t="e">
@@ -3531,20 +3552,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" t="e">
+      <c r="AR23" t="e" s="0">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>160</v>
       </c>
       <c r="AW23" s="48">
@@ -3583,10 +3604,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO23" s="48" t="e">
@@ -3643,14 +3664,14 @@
       <c r="F31" s="46">
         <v>2</v>
       </c>
-      <c r="G31" t="s">
+      <c r="G31" t="s" s="0">
         <v>128</v>
       </c>
       <c r="H31" s="46">
         <f>F31*G31</f>
         <v>600</v>
       </c>
-      <c r="I31" t="s">
+      <c r="I31" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J31" s="46">
@@ -3778,20 +3799,20 @@
       <c r="AQ31" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR31">
+      <c r="AR31" s="0">
         <f>ROUND(AN31+AO31+AP31,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS31" t="s">
+      <c r="AS31" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT31" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU31" t="s">
+      <c r="AU31" t="s" s="0">
         <v>162</v>
       </c>
-      <c r="AV31" t="s">
+      <c r="AV31" t="s" s="0">
         <v>167</v>
       </c>
       <c r="AW31" s="48">
@@ -3830,10 +3851,10 @@
       <c r="BL31" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM31" t="s">
+      <c r="BM31" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN31" t="s">
+      <c r="BN31" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO31" s="48">
@@ -3868,14 +3889,14 @@
       <c r="F32" s="46">
         <v>2</v>
       </c>
-      <c r="G32" t="s">
+      <c r="G32" t="s" s="0">
         <v>129</v>
       </c>
       <c r="H32" s="46">
         <f>F32*G32</f>
         <v>800</v>
       </c>
-      <c r="I32" t="s">
+      <c r="I32" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J32" s="46">
@@ -4003,20 +4024,20 @@
       <c r="AQ32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR32">
+      <c r="AR32" s="0">
         <f>ROUND(AN32+AO32+AP32,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS32" t="s">
+      <c r="AS32" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT32" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU32" t="s">
+      <c r="AU32" t="s" s="0">
         <v>168</v>
       </c>
-      <c r="AV32" t="s">
+      <c r="AV32" t="s" s="0">
         <v>169</v>
       </c>
       <c r="AW32" s="48">
@@ -4055,10 +4076,10 @@
       <c r="BL32" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM32" t="s">
+      <c r="BM32" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN32" t="s">
+      <c r="BN32" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO32" s="48">
@@ -4093,14 +4114,14 @@
       <c r="F33" s="46">
         <v>2</v>
       </c>
-      <c r="G33" t="s">
+      <c r="G33" t="s" s="0">
         <v>161</v>
       </c>
       <c r="H33" s="46">
         <f>F33*G33</f>
         <v>1000</v>
       </c>
-      <c r="I33" t="s">
+      <c r="I33" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J33" s="46">
@@ -4228,20 +4249,20 @@
       <c r="AQ33" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR33">
+      <c r="AR33" s="0">
         <f>ROUND(AN33+AO33+AP33,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS33" t="s">
+      <c r="AS33" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT33" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU33" t="s">
+      <c r="AU33" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV33" t="s">
+      <c r="AV33" t="s" s="0">
         <v>170</v>
       </c>
       <c r="AW33" s="48">
@@ -4280,10 +4301,10 @@
       <c r="BL33" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM33" t="s">
+      <c r="BM33" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN33" t="s">
+      <c r="BN33" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO33" s="48">
@@ -4319,14 +4340,14 @@
       <c r="F35" s="46">
         <v>2</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G35" t="s" s="0">
         <v>128</v>
       </c>
       <c r="H35" s="46">
         <f>F35*G35</f>
         <v>600</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I35" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J35" s="46">
@@ -4454,20 +4475,20 @@
       <c r="AQ35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR35">
+      <c r="AR35" s="0">
         <f>ROUND(AN35+AO35+AP35,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS35" t="s">
+      <c r="AS35" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT35" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU35" t="s">
+      <c r="AU35" t="s" s="0">
         <v>171</v>
       </c>
-      <c r="AV35" t="s">
+      <c r="AV35" t="s" s="0">
         <v>172</v>
       </c>
       <c r="AW35" s="48">
@@ -4506,10 +4527,10 @@
       <c r="BL35" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM35" t="s">
+      <c r="BM35" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN35" t="s">
+      <c r="BN35" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO35" s="48">
@@ -4544,14 +4565,14 @@
       <c r="F36" s="46">
         <v>2</v>
       </c>
-      <c r="G36" t="s">
+      <c r="G36" t="s" s="0">
         <v>129</v>
       </c>
       <c r="H36" s="46">
         <f>F36*G36</f>
         <v>800</v>
       </c>
-      <c r="I36" t="s">
+      <c r="I36" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J36" s="46">
@@ -4679,20 +4700,20 @@
       <c r="AQ36" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR36">
+      <c r="AR36" s="0">
         <f>ROUND(AN36+AO36+AP36,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS36" t="s">
+      <c r="AS36" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT36" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU36" t="s">
+      <c r="AU36" t="s" s="0">
         <v>173</v>
       </c>
-      <c r="AV36" t="s">
+      <c r="AV36" t="s" s="0">
         <v>174</v>
       </c>
       <c r="AW36" s="48">
@@ -4731,10 +4752,10 @@
       <c r="BL36" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM36" t="s">
+      <c r="BM36" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN36" t="s">
+      <c r="BN36" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO36" s="48">
@@ -4769,14 +4790,14 @@
       <c r="F37" s="46">
         <v>2</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G37" t="s" s="0">
         <v>161</v>
       </c>
       <c r="H37" s="46">
         <f>F37*G37</f>
         <v>1000</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I37" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J37" s="46">
@@ -4904,20 +4925,20 @@
       <c r="AQ37" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR37">
+      <c r="AR37" s="0">
         <f>ROUND(AN37+AO37+AP37,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS37" t="s">
+      <c r="AS37" t="s" s="0">
         <v>107</v>
       </c>
       <c r="AT37" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU37" t="s">
+      <c r="AU37" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV37" t="s">
+      <c r="AV37" t="s" s="0">
         <v>170</v>
       </c>
       <c r="AW37" s="48">
@@ -4956,10 +4977,10 @@
       <c r="BL37" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM37" t="s">
+      <c r="BM37" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN37" t="s">
+      <c r="BN37" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO37" s="48">
@@ -4985,34 +5006,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -6538,14 +6559,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -6673,20 +6694,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>158</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>177</v>
       </c>
       <c r="AW23" s="48">
@@ -6725,10 +6746,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>178</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>131</v>
       </c>
       <c r="BO23" s="48">
@@ -6904,32 +6925,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -8455,14 +8476,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -8590,11 +8611,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -8806,34 +8827,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -10359,14 +10380,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -10494,20 +10515,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>132</v>
       </c>
       <c r="AW23" s="48">
@@ -10546,10 +10567,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO23" s="48">
@@ -10724,34 +10745,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -12277,14 +12298,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -12412,20 +12433,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>164</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -12464,10 +12485,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>163</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -12642,32 +12663,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -14193,14 +14214,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -14328,11 +14349,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -14543,34 +14564,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -16096,14 +16117,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -16231,20 +16252,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>164</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -16283,10 +16304,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>163</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -16461,32 +16482,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -18012,14 +18033,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -18147,11 +18168,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -18362,34 +18383,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -19915,14 +19936,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -20050,20 +20071,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>189</v>
       </c>
       <c r="AW23" s="48">
@@ -20102,10 +20123,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>195</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>194</v>
       </c>
       <c r="BO23" s="48">
@@ -20280,32 +20301,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -21831,14 +21852,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -21966,11 +21987,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -22181,34 +22202,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -23869,20 +23890,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>175</v>
       </c>
       <c r="AW23" s="48">
@@ -23921,10 +23942,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>175</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>176</v>
       </c>
       <c r="BO23" s="48">
@@ -24096,34 +24117,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -25784,20 +25805,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -25836,10 +25857,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>155</v>
       </c>
       <c r="BO23" s="48">
@@ -26012,34 +26033,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -27700,20 +27721,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>175</v>
       </c>
       <c r="AW23" s="48">
@@ -27752,10 +27773,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>175</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>196</v>
       </c>
       <c r="BO23" s="48">
@@ -27927,32 +27948,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -29478,14 +29499,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -29613,11 +29634,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -29828,34 +29849,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -31381,14 +31402,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -31516,20 +31537,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>570.48</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>191</v>
       </c>
       <c r="AW23" s="16">
@@ -31568,10 +31589,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>198</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>197</v>
       </c>
       <c r="BO23" s="48">
@@ -31743,34 +31764,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -33296,14 +33317,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -33431,20 +33452,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>558.96</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>191</v>
       </c>
       <c r="AW23" s="48">
@@ -33483,10 +33504,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>200</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>199</v>
       </c>
       <c r="BO23" s="48">
@@ -33658,32 +33679,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -35209,14 +35230,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -35344,11 +35365,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>188.22</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -35559,34 +35580,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -37112,14 +37133,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -37247,20 +37268,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>564.66</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>191</v>
       </c>
       <c r="AW23" s="16">
@@ -37299,10 +37320,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>191</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>193</v>
       </c>
       <c r="BO23" s="48">
@@ -37477,34 +37498,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -39030,14 +39051,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -39165,20 +39186,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>564.66</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>191</v>
       </c>
       <c r="AW23" s="16">
@@ -39217,10 +39238,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>191</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>192</v>
       </c>
       <c r="BO23" s="48">
@@ -39395,32 +39416,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -40946,14 +40967,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -41081,11 +41102,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -41296,34 +41317,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -42984,20 +43005,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>28.23</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>209</v>
       </c>
       <c r="AW23" s="66">
@@ -43036,10 +43057,10 @@
       <c r="BL23" s="66" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>210</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>211</v>
       </c>
       <c r="BO23" s="66">
@@ -43211,34 +43232,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -44899,20 +44920,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="66">
@@ -44951,10 +44972,10 @@
       <c r="BL23" s="66" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>212</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>213</v>
       </c>
       <c r="BO23" s="66">
@@ -45124,20 +45145,20 @@
       <c r="AQ24" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR24">
+      <c r="AR24" s="0">
         <f>ROUND(AN24+AO24+AP24,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS24" t="s">
+      <c r="AS24" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT24" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU24" t="s">
+      <c r="AU24" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV24" t="s">
+      <c r="AV24" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW24" s="66">
@@ -45176,10 +45197,10 @@
       <c r="BL24" s="66" t="s">
         <v>148</v>
       </c>
-      <c r="BM24" t="s">
+      <c r="BM24" t="s" s="0">
         <v>215</v>
       </c>
-      <c r="BN24" t="s">
+      <c r="BN24" t="s" s="0">
         <v>216</v>
       </c>
       <c r="BO24" s="66">
@@ -45351,36 +45372,36 @@
   <dimension ref="A1:BU25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="18" max="18" width="14.85546875" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
-    <col min="71" max="71" width="22.140625" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="18" max="18" customWidth="true" width="14.85546875"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="71" max="71" customWidth="true" width="22.140625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -47051,20 +47072,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -47103,10 +47124,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23">
+      <c r="BM23" s="0">
         <v>292.60462000000001</v>
       </c>
-      <c r="BN23">
+      <c r="BN23" s="0">
         <v>682</v>
       </c>
       <c r="BO23" s="48">
@@ -47288,35 +47309,35 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="64" max="64" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="64" max="64" bestFit="true" customWidth="true" width="10.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -48977,20 +48998,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="66">
@@ -49029,10 +49050,10 @@
       <c r="BL23" s="66" t="s">
         <v>217</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>218</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>173</v>
       </c>
       <c r="BO23" s="66">
@@ -49204,35 +49225,35 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="64" max="64" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="64" max="64" bestFit="true" customWidth="true" width="10.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -50893,20 +50914,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="66">
@@ -50945,10 +50966,10 @@
       <c r="BL23" s="66" t="s">
         <v>217</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>219</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>220</v>
       </c>
       <c r="BO23" s="66">
@@ -51118,20 +51139,20 @@
       <c r="AQ24" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR24">
+      <c r="AR24" s="0">
         <f>ROUND(AN24+AO24+AP24,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS24" t="s">
+      <c r="AS24" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT24" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU24" t="s">
+      <c r="AU24" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV24" t="s">
+      <c r="AV24" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW24" s="66">
@@ -51170,10 +51191,10 @@
       <c r="BL24" s="66" t="s">
         <v>217</v>
       </c>
-      <c r="BM24" t="s">
+      <c r="BM24" t="s" s="0">
         <v>221</v>
       </c>
-      <c r="BN24" t="s">
+      <c r="BN24" t="s" s="0">
         <v>222</v>
       </c>
       <c r="BO24" s="66">
@@ -51345,34 +51366,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -53033,20 +53054,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="66">
@@ -53085,11 +53106,11 @@
       <c r="BL23" s="66" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>219</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>220</v>
+      <c r="BM23" t="s" s="0">
+        <v>228</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>227</v>
       </c>
       <c r="BO23" s="66">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -53258,20 +53279,20 @@
       <c r="AQ24" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR24">
+      <c r="AR24" s="0">
         <f>ROUND(AN24+AO24+AP24,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS24" t="s">
+      <c r="AS24" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT24" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU24" t="s">
+      <c r="AU24" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV24" t="s">
+      <c r="AV24" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW24" s="66">
@@ -53310,11 +53331,11 @@
       <c r="BL24" s="66" t="s">
         <v>148</v>
       </c>
-      <c r="BM24" t="s">
-        <v>221</v>
-      </c>
-      <c r="BN24" t="s">
-        <v>222</v>
+      <c r="BM24" t="s" s="0">
+        <v>229</v>
+      </c>
+      <c r="BN24" t="s" s="0">
+        <v>213</v>
       </c>
       <c r="BO24" s="66">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -53485,37 +53506,37 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="18" max="18" width="11.28515625" customWidth="1"/>
-    <col min="19" max="19" width="11.140625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="23.85546875" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="50" max="50" width="11" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="18" max="18" customWidth="true" width="11.28515625"/>
+    <col min="19" max="19" customWidth="true" width="11.140625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="23.85546875"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="50" max="50" customWidth="true" width="11.0"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -55044,14 +55065,14 @@
       <c r="F23" s="46">
         <v>5</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>128</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>1000</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -55179,20 +55200,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.31800000000001</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>189</v>
       </c>
       <c r="AW23" s="48">
@@ -55231,10 +55252,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>208</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>207</v>
       </c>
       <c r="BO23" s="48">
@@ -55410,34 +55431,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -56966,7 +56987,7 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23">
+      <c r="G23" s="0">
         <v>300</v>
       </c>
       <c r="H23" s="46">
@@ -57101,20 +57122,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -57153,11 +57174,11 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
-        <v>206</v>
-      </c>
-      <c r="BN23" t="s">
-        <v>205</v>
+      <c r="BM23" t="s" s="0">
+        <v>226</v>
+      </c>
+      <c r="BN23" t="s" s="0">
+        <v>225</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -57332,32 +57353,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -59018,20 +59039,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -59070,10 +59091,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>149</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>164</v>
       </c>
       <c r="BO23" s="48">
@@ -59248,32 +59269,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -60934,11 +60955,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -61149,34 +61170,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
+    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -62702,14 +62723,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -62837,20 +62858,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s">
+      <c r="AU23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="AV23" t="s">
+      <c r="AV23" t="s" s="0">
         <v>189</v>
       </c>
       <c r="AW23" s="48">
@@ -62889,10 +62910,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s">
+      <c r="BM23" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="BN23" t="s">
+      <c r="BN23" t="s" s="0">
         <v>108</v>
       </c>
       <c r="BO23" s="48">
@@ -63065,32 +63086,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="80.42578125" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="8.28515625" customWidth="1"/>
-    <col min="7" max="7" width="10.140625" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" customWidth="1"/>
-    <col min="11" max="11" width="6.28515625" customWidth="1"/>
-    <col min="29" max="29" width="10.28515625" customWidth="1"/>
-    <col min="30" max="30" width="12.85546875" customWidth="1"/>
-    <col min="31" max="31" width="8.7109375" customWidth="1"/>
-    <col min="35" max="35" width="14.28515625" customWidth="1"/>
-    <col min="43" max="43" width="11.85546875" customWidth="1"/>
-    <col min="44" max="44" width="23.28515625" customWidth="1"/>
-    <col min="46" max="46" width="11.85546875" customWidth="1"/>
-    <col min="47" max="47" width="15.28515625" customWidth="1"/>
-    <col min="48" max="48" width="20.28515625" customWidth="1"/>
-    <col min="49" max="49" width="11.42578125" customWidth="1"/>
-    <col min="51" max="51" width="13.85546875" customWidth="1"/>
-    <col min="60" max="60" width="12.5703125" customWidth="1"/>
-    <col min="61" max="61" width="21.7109375" customWidth="1"/>
-    <col min="62" max="63" width="30.5703125" customWidth="1"/>
-    <col min="65" max="65" width="41.140625" customWidth="1"/>
-    <col min="66" max="66" width="37" customWidth="1"/>
-    <col min="67" max="67" width="18.85546875" customWidth="1"/>
-    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="2" max="2" customWidth="true" width="26.85546875"/>
+    <col min="3" max="3" customWidth="true" width="19.28515625"/>
+    <col min="4" max="4" customWidth="true" width="80.42578125"/>
+    <col min="5" max="5" customWidth="true" width="10.42578125"/>
+    <col min="6" max="6" customWidth="true" width="8.28515625"/>
+    <col min="7" max="7" customWidth="true" width="10.140625"/>
+    <col min="8" max="8" customWidth="true" width="11.85546875"/>
+    <col min="11" max="11" customWidth="true" width="6.28515625"/>
+    <col min="29" max="29" customWidth="true" width="10.28515625"/>
+    <col min="30" max="30" customWidth="true" width="12.85546875"/>
+    <col min="31" max="31" customWidth="true" width="8.7109375"/>
+    <col min="35" max="35" customWidth="true" width="14.28515625"/>
+    <col min="43" max="43" customWidth="true" width="11.85546875"/>
+    <col min="44" max="44" customWidth="true" width="23.28515625"/>
+    <col min="46" max="46" customWidth="true" width="11.85546875"/>
+    <col min="47" max="47" customWidth="true" width="15.28515625"/>
+    <col min="48" max="48" customWidth="true" width="20.28515625"/>
+    <col min="49" max="49" customWidth="true" width="11.42578125"/>
+    <col min="51" max="51" customWidth="true" width="13.85546875"/>
+    <col min="60" max="60" customWidth="true" width="12.5703125"/>
+    <col min="61" max="61" customWidth="true" width="21.7109375"/>
+    <col min="62" max="63" customWidth="true" width="30.5703125"/>
+    <col min="65" max="65" customWidth="true" width="41.140625"/>
+    <col min="66" max="66" customWidth="true" width="37.0"/>
+    <col min="67" max="67" customWidth="true" width="18.85546875"/>
+    <col min="68" max="68" customWidth="true" width="34.42578125"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -64616,14 +64637,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" t="s" s="0">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" t="s" s="0">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -64751,11 +64772,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23">
+      <c r="AR23" s="0">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s">
+      <c r="AS23" t="s" s="0">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">

</xml_diff>

<commit_message>
Fixes For The Failed Test Scenarios Of Bank Payment Screens
Fixes For The Failed Test Scenarios Of Bank Payment Screens
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="29" activeTab="29"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="5" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5903" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6094" uniqueCount="324">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -680,19 +680,10 @@
     <t>712</t>
   </si>
   <si>
-    <t>266.61192</t>
-  </si>
-  <si>
     <t>386</t>
   </si>
   <si>
     <t>ROAU-RM-KDK-02</t>
-  </si>
-  <si>
-    <t>261.53222</t>
-  </si>
-  <si>
-    <t>144</t>
   </si>
   <si>
     <t>RM WH 50</t>
@@ -711,12 +702,6 @@
   </si>
   <si>
     <t>294</t>
-  </si>
-  <si>
-    <t>1104</t>
-  </si>
-  <si>
-    <t>879.88404</t>
   </si>
   <si>
     <t>1106</t>
@@ -785,16 +770,268 @@
     <t>186.49443</t>
   </si>
   <si>
-    <t>7209</t>
-  </si>
-  <si>
-    <t>186.49927</t>
-  </si>
-  <si>
     <t>7214</t>
   </si>
   <si>
     <t>186.49914</t>
+  </si>
+  <si>
+    <t>23998.05</t>
+  </si>
+  <si>
+    <t>4124</t>
+  </si>
+  <si>
+    <t>1378.33564</t>
+  </si>
+  <si>
+    <t>1354</t>
+  </si>
+  <si>
+    <t>3422.47109</t>
+  </si>
+  <si>
+    <t>2399.55</t>
+  </si>
+  <si>
+    <t>4126</t>
+  </si>
+  <si>
+    <t>1378.83065</t>
+  </si>
+  <si>
+    <t>4128</t>
+  </si>
+  <si>
+    <t>1379.32518</t>
+  </si>
+  <si>
+    <t>4130</t>
+  </si>
+  <si>
+    <t>1379.81924</t>
+  </si>
+  <si>
+    <t>4132</t>
+  </si>
+  <si>
+    <t>1380.31282</t>
+  </si>
+  <si>
+    <t>4134</t>
+  </si>
+  <si>
+    <t>1380.80592</t>
+  </si>
+  <si>
+    <t>4136</t>
+  </si>
+  <si>
+    <t>1381.29854</t>
+  </si>
+  <si>
+    <t>4138</t>
+  </si>
+  <si>
+    <t>1381.79069</t>
+  </si>
+  <si>
+    <t>4142</t>
+  </si>
+  <si>
+    <t>1380.72892</t>
+  </si>
+  <si>
+    <t>4144</t>
+  </si>
+  <si>
+    <t>1381.22063</t>
+  </si>
+  <si>
+    <t>4146</t>
+  </si>
+  <si>
+    <t>1381.71186</t>
+  </si>
+  <si>
+    <t>4148</t>
+  </si>
+  <si>
+    <t>1382.20262</t>
+  </si>
+  <si>
+    <t>4150</t>
+  </si>
+  <si>
+    <t>1382.69291</t>
+  </si>
+  <si>
+    <t>4152</t>
+  </si>
+  <si>
+    <t>1383.18273</t>
+  </si>
+  <si>
+    <t>4156</t>
+  </si>
+  <si>
+    <t>1383.09587</t>
+  </si>
+  <si>
+    <t>4160</t>
+  </si>
+  <si>
+    <t>1383.00918</t>
+  </si>
+  <si>
+    <t>4166</t>
+  </si>
+  <si>
+    <t>1382.3482</t>
+  </si>
+  <si>
+    <t>4168</t>
+  </si>
+  <si>
+    <t>1382.8363</t>
+  </si>
+  <si>
+    <t>4170</t>
+  </si>
+  <si>
+    <t>1383.32393</t>
+  </si>
+  <si>
+    <t>4172</t>
+  </si>
+  <si>
+    <t>1383.81109</t>
+  </si>
+  <si>
+    <t>4174</t>
+  </si>
+  <si>
+    <t>1384.29779</t>
+  </si>
+  <si>
+    <t>4176</t>
+  </si>
+  <si>
+    <t>1384.78402</t>
+  </si>
+  <si>
+    <t>4178</t>
+  </si>
+  <si>
+    <t>1385.26979</t>
+  </si>
+  <si>
+    <t>4180</t>
+  </si>
+  <si>
+    <t>1385.75509</t>
+  </si>
+  <si>
+    <t>4182</t>
+  </si>
+  <si>
+    <t>1386.23993</t>
+  </si>
+  <si>
+    <t>4184</t>
+  </si>
+  <si>
+    <t>1386.7243</t>
+  </si>
+  <si>
+    <t>4186</t>
+  </si>
+  <si>
+    <t>1387.20821</t>
+  </si>
+  <si>
+    <t>4188</t>
+  </si>
+  <si>
+    <t>1387.69166</t>
+  </si>
+  <si>
+    <t>4190</t>
+  </si>
+  <si>
+    <t>1388.17465</t>
+  </si>
+  <si>
+    <t>4192</t>
+  </si>
+  <si>
+    <t>1387.64705</t>
+  </si>
+  <si>
+    <t>4194</t>
+  </si>
+  <si>
+    <t>1388.1296</t>
+  </si>
+  <si>
+    <t>4196</t>
+  </si>
+  <si>
+    <t>1388.61169</t>
+  </si>
+  <si>
+    <t>4198</t>
+  </si>
+  <si>
+    <t>1389.09332</t>
+  </si>
+  <si>
+    <t>4200</t>
+  </si>
+  <si>
+    <t>1389.57449</t>
+  </si>
+  <si>
+    <t>4202</t>
+  </si>
+  <si>
+    <t>1390.0552</t>
+  </si>
+  <si>
+    <t>4204</t>
+  </si>
+  <si>
+    <t>1390.53545</t>
+  </si>
+  <si>
+    <t>4206</t>
+  </si>
+  <si>
+    <t>1391.01525</t>
+  </si>
+  <si>
+    <t>4208</t>
+  </si>
+  <si>
+    <t>1391.49459</t>
+  </si>
+  <si>
+    <t>4210</t>
+  </si>
+  <si>
+    <t>1390.96767</t>
+  </si>
+  <si>
+    <t>4212</t>
+  </si>
+  <si>
+    <t>1390.44125</t>
+  </si>
+  <si>
+    <t>4216</t>
+  </si>
+  <si>
+    <t>1391.39866</t>
   </si>
 </sst>
 </file>
@@ -37349,7 +37586,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -37388,10 +37625,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>232</v>
+        <v>227</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -46745,7 +46982,7 @@
         <v>201</v>
       </c>
       <c r="BU22" s="97" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:73" ht="15.75" thickBot="1">
@@ -46982,7 +47219,7 @@
         <v>3</v>
       </c>
       <c r="BU23" t="s" s="0">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:73" ht="15.75" thickBot="1">
@@ -48844,7 +49081,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>203</v>
+        <v>243</v>
       </c>
       <c r="AW23" s="66">
         <f>AM23</f>
@@ -48883,10 +49120,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>204</v>
+        <v>323</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>205</v>
+        <v>322</v>
       </c>
       <c r="BO23" s="66">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -50759,7 +50996,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>149</v>
+        <v>243</v>
       </c>
       <c r="AW23" s="66">
         <f>AM23</f>
@@ -50798,10 +51035,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>206</v>
+        <v>283</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>207</v>
+        <v>282</v>
       </c>
       <c r="BO23" s="66">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -50821,10 +51058,10 @@
         <v>2</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D24" s="94" t="s">
         <v>12</v>
@@ -50984,7 +51221,7 @@
         <v>108</v>
       </c>
       <c r="AV24" t="s" s="0">
-        <v>149</v>
+        <v>238</v>
       </c>
       <c r="AW24" s="66">
         <f>AM24</f>
@@ -51023,10 +51260,10 @@
         <v>148</v>
       </c>
       <c r="BM24" t="s" s="0">
-        <v>209</v>
+        <v>242</v>
       </c>
       <c r="BN24" t="s" s="0">
-        <v>210</v>
+        <v>241</v>
       </c>
       <c r="BO24" s="66">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -52936,10 +53173,10 @@
       <c r="BH23" s="3"/>
       <c r="BI23" s="66"/>
       <c r="BL23" s="66" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="BN23" t="s" s="0">
         <v>173</v>
@@ -54852,13 +55089,13 @@
       <c r="BH23" s="3"/>
       <c r="BI23" s="66"/>
       <c r="BL23" s="66" t="s">
+        <v>208</v>
+      </c>
+      <c r="BM23" t="s" s="0">
+        <v>210</v>
+      </c>
+      <c r="BN23" t="s" s="0">
         <v>211</v>
-      </c>
-      <c r="BM23" t="s" s="0">
-        <v>213</v>
-      </c>
-      <c r="BN23" t="s" s="0">
-        <v>214</v>
       </c>
       <c r="BO23" s="66">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -54878,10 +55115,10 @@
         <v>2</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D24" s="94" t="s">
         <v>12</v>
@@ -55077,13 +55314,13 @@
       <c r="BH24" s="3"/>
       <c r="BI24" s="66"/>
       <c r="BL24" s="66" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="BM24" t="s" s="0">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="BN24" t="s" s="0">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="BO24" s="66">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -56995,10 +57232,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="BO23" s="66">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -57018,10 +57255,10 @@
         <v>2</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D24" s="94" t="s">
         <v>12</v>
@@ -57220,10 +57457,10 @@
         <v>148</v>
       </c>
       <c r="BM24" t="s" s="0">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="BN24" t="s" s="0">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="BO24" s="66">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -58939,7 +59176,7 @@
         <v>201</v>
       </c>
       <c r="BU22" s="97" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="23" spans="1:73" ht="15.75" thickBot="1">
@@ -59176,7 +59413,7 @@
         <v>3</v>
       </c>
       <c r="BU23" t="s" s="0">
-        <v>223</v>
+        <v>218</v>
       </c>
     </row>
     <row r="24" spans="1:73" ht="15.75" thickBot="1">
@@ -60886,31 +61123,31 @@
         <v>201</v>
       </c>
       <c r="BU22" s="97" t="s">
+        <v>217</v>
+      </c>
+      <c r="BV22" s="90" t="s">
+        <v>219</v>
+      </c>
+      <c r="BW22" s="90" t="s">
+        <v>220</v>
+      </c>
+      <c r="BX22" s="90" t="s">
+        <v>221</v>
+      </c>
+      <c r="BY22" s="90" t="s">
         <v>222</v>
       </c>
-      <c r="BV22" s="90" t="s">
+      <c r="BZ22" s="90" t="s">
+        <v>223</v>
+      </c>
+      <c r="CA22" s="90" t="s">
         <v>224</v>
       </c>
-      <c r="BW22" s="90" t="s">
-        <v>225</v>
-      </c>
-      <c r="BX22" s="90" t="s">
-        <v>226</v>
-      </c>
-      <c r="BY22" s="90" t="s">
-        <v>227</v>
-      </c>
-      <c r="BZ22" s="90" t="s">
-        <v>228</v>
-      </c>
-      <c r="CA22" s="90" t="s">
-        <v>229</v>
-      </c>
       <c r="CB22" s="90" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="CC22" s="90" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="23" spans="1:81" ht="15.75" thickBot="1">
@@ -61081,7 +61318,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="AW23" s="66">
         <f>AM23</f>
@@ -61120,10 +61357,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="BO23" s="66">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -61147,16 +61384,16 @@
         <v>3</v>
       </c>
       <c r="BU23" t="s" s="0">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="BV23" t="s" s="0">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="BW23" t="s" s="0">
-        <v>235</v>
+        <v>230</v>
       </c>
       <c r="BX23" t="s" s="0">
-        <v>236</v>
+        <v>231</v>
       </c>
       <c r="BY23" t="s" s="0">
         <v>109</v>
@@ -62882,31 +63119,31 @@
         <v>201</v>
       </c>
       <c r="BU22" s="97" t="s">
+        <v>217</v>
+      </c>
+      <c r="BV22" s="90" t="s">
+        <v>219</v>
+      </c>
+      <c r="BW22" s="90" t="s">
+        <v>220</v>
+      </c>
+      <c r="BX22" s="90" t="s">
+        <v>221</v>
+      </c>
+      <c r="BY22" s="90" t="s">
         <v>222</v>
       </c>
-      <c r="BV22" s="90" t="s">
+      <c r="BZ22" s="90" t="s">
+        <v>223</v>
+      </c>
+      <c r="CA22" s="90" t="s">
         <v>224</v>
       </c>
-      <c r="BW22" s="90" t="s">
-        <v>225</v>
-      </c>
-      <c r="BX22" s="90" t="s">
-        <v>226</v>
-      </c>
-      <c r="BY22" s="90" t="s">
-        <v>227</v>
-      </c>
-      <c r="BZ22" s="90" t="s">
-        <v>228</v>
-      </c>
-      <c r="CA22" s="90" t="s">
-        <v>229</v>
-      </c>
       <c r="CB22" s="90" t="s">
-        <v>237</v>
+        <v>232</v>
       </c>
       <c r="CC22" s="90" t="s">
-        <v>238</v>
+        <v>233</v>
       </c>
     </row>
     <row r="23" spans="1:81" ht="15.75" thickBot="1">
@@ -63077,7 +63314,7 @@
         <v>108</v>
       </c>
       <c r="AV23" t="s" s="0">
-        <v>234</v>
+        <v>229</v>
       </c>
       <c r="AW23" s="48">
         <f>AM23</f>
@@ -63116,10 +63353,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>244</v>
+        <v>237</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>243</v>
+        <v>236</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -63143,13 +63380,13 @@
         <v>3</v>
       </c>
       <c r="BU23" t="s" s="0">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="BV23" s="75" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="BW23" s="75" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
       <c r="BX23" s="75">
         <v>5</v>
@@ -65083,10 +65320,10 @@
         <v>148</v>
       </c>
       <c r="BM23" t="s" s="0">
-        <v>218</v>
+        <v>319</v>
       </c>
       <c r="BN23" t="s" s="0">
-        <v>217</v>
+        <v>318</v>
       </c>
       <c r="BO23" s="48">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>

</xml_diff>

<commit_message>
Fixes For The Failed Test Scenarios Of Adv SO
Fixes For The Failed Test Scenarios Of Adv SO
</commit_message>
<xml_diff>
--- a/testdata/DirectGrnDetails.xlsx
+++ b/testdata/DirectGrnDetails.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="4" lowestEdited="5" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915" firstSheet="2" activeTab="5"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6915"/>
   </bookViews>
   <sheets>
     <sheet name="DirectGrnGenUD" sheetId="38" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5922" uniqueCount="253">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5890" uniqueCount="245">
   <si>
     <t>Scenario  : Local Purchase - Stock UOM and Purchase UOM (Similar)</t>
   </si>
@@ -737,12 +737,6 @@
     <t>186.49914</t>
   </si>
   <si>
-    <t>4270</t>
-  </si>
-  <si>
-    <t>1382.06151</t>
-  </si>
-  <si>
     <t>386</t>
   </si>
   <si>
@@ -794,34 +788,16 @@
     <t>2399.55</t>
   </si>
   <si>
-    <t>4224</t>
-  </si>
-  <si>
-    <t>1393.30804</t>
-  </si>
-  <si>
-    <t>4272</t>
-  </si>
-  <si>
-    <t>1382.53786</t>
-  </si>
-  <si>
-    <t>4274</t>
-  </si>
-  <si>
-    <t>1383.01377</t>
-  </si>
-  <si>
     <t>4276</t>
   </si>
   <si>
     <t>1383.48923</t>
   </si>
   <si>
-    <t>4278</t>
+    <t>4282</t>
   </si>
   <si>
-    <t>1383.96425</t>
+    <t>1382.93517</t>
   </si>
 </sst>
 </file>
@@ -1862,44 +1838,44 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="99" width="9.0"/>
-    <col min="2" max="2" customWidth="true" style="99" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" style="99" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" style="99" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" style="99" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" style="99" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" style="99" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" style="99" width="11.85546875"/>
-    <col min="9" max="10" style="99" width="9.0"/>
-    <col min="11" max="11" customWidth="true" style="99" width="6.28515625"/>
-    <col min="12" max="28" style="99" width="9.0"/>
-    <col min="29" max="29" customWidth="true" style="99" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" style="99" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" style="99" width="8.7109375"/>
-    <col min="32" max="34" style="99" width="9.0"/>
-    <col min="35" max="35" customWidth="true" style="99" width="14.28515625"/>
-    <col min="36" max="42" style="99" width="9.0"/>
-    <col min="43" max="43" customWidth="true" style="99" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" style="99" width="23.28515625"/>
-    <col min="45" max="45" style="99" width="9.0"/>
-    <col min="46" max="46" customWidth="true" style="99" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" style="99" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" style="99" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" style="99" width="11.42578125"/>
-    <col min="50" max="50" style="99" width="9.0"/>
-    <col min="51" max="51" customWidth="true" style="99" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" style="99" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" style="99" width="19.0"/>
-    <col min="54" max="59" style="99" width="9.0"/>
-    <col min="60" max="60" customWidth="true" style="99" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" style="99" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" style="99" width="30.5703125"/>
-    <col min="64" max="64" style="99" width="9.0"/>
-    <col min="65" max="65" customWidth="true" style="99" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" style="99" width="37.0"/>
-    <col min="67" max="67" customWidth="true" style="99" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" style="99" width="34.42578125"/>
-    <col min="69" max="16384" style="99" width="9.0"/>
+    <col min="1" max="1" width="9" style="99"/>
+    <col min="2" max="2" width="26.85546875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" style="99" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="99" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="99" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="99" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="99" customWidth="1"/>
+    <col min="9" max="10" width="9" style="99"/>
+    <col min="11" max="11" width="6.28515625" style="99" customWidth="1"/>
+    <col min="12" max="28" width="9" style="99"/>
+    <col min="29" max="29" width="10.28515625" style="99" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" style="99" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="99" customWidth="1"/>
+    <col min="32" max="34" width="9" style="99"/>
+    <col min="35" max="35" width="14.28515625" style="99" customWidth="1"/>
+    <col min="36" max="42" width="9" style="99"/>
+    <col min="43" max="43" width="11.85546875" style="99" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" style="99" customWidth="1"/>
+    <col min="45" max="45" width="9" style="99"/>
+    <col min="46" max="46" width="11.85546875" style="99" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="99" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" style="99" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" style="99" customWidth="1"/>
+    <col min="50" max="50" width="9" style="99"/>
+    <col min="51" max="51" width="13.85546875" style="99" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" style="99" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" style="99" bestFit="1" customWidth="1"/>
+    <col min="54" max="59" width="9" style="99"/>
+    <col min="60" max="60" width="12.5703125" style="99" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" style="99" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" style="99" customWidth="1"/>
+    <col min="64" max="64" width="9" style="99"/>
+    <col min="65" max="65" width="41.140625" style="99" customWidth="1"/>
+    <col min="66" max="66" width="37" style="99" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" style="99" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" style="99" customWidth="1"/>
+    <col min="69" max="16384" width="9" style="99"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -3573,11 +3549,11 @@
       <c r="AT23" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="99">
+      <c r="AU23" s="99" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="99">
-        <v>242</v>
+      <c r="AV23" s="99" t="s">
+        <v>149</v>
       </c>
       <c r="AW23" s="112">
         <f>AM23</f>
@@ -3615,11 +3591,11 @@
       <c r="BL23" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="99">
-        <v>252</v>
-      </c>
-      <c r="BN23" t="s" s="99">
-        <v>251</v>
+      <c r="BM23" s="99" t="s">
+        <v>244</v>
+      </c>
+      <c r="BN23" s="99" t="s">
+        <v>243</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -3794,36 +3770,36 @@
   <dimension ref="A1:BU25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="18" max="18" customWidth="true" width="14.85546875"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
-    <col min="71" max="71" customWidth="true" width="22.140625"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="71" max="71" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -5496,20 +5472,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -5548,10 +5524,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" s="0">
+      <c r="BM23">
         <v>292.60462000000001</v>
       </c>
-      <c r="BN23" s="0">
+      <c r="BN23">
         <v>682</v>
       </c>
       <c r="BO23" s="48">
@@ -5575,7 +5551,7 @@
       <c r="BT23" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="BU23" t="s" s="0">
+      <c r="BU23" t="s">
         <v>204</v>
       </c>
     </row>
@@ -5736,41 +5712,41 @@
   <dimension ref="A1:CC25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="18" max="18" customWidth="true" width="11.28515625"/>
-    <col min="19" max="19" customWidth="true" width="11.140625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="23.85546875"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="50" max="50" customWidth="true" width="11.0"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
-    <col min="74" max="74" bestFit="true" customWidth="true" width="12.85546875"/>
-    <col min="75" max="75" bestFit="true" customWidth="true" width="9.140625"/>
-    <col min="78" max="78" bestFit="true" customWidth="true" width="17.5703125"/>
-    <col min="79" max="79" bestFit="true" customWidth="true" width="14.0"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="18" max="18" width="11.28515625" customWidth="1"/>
+    <col min="19" max="19" width="11.140625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="23.85546875" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="50" max="50" width="11" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="74" max="74" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="75" max="75" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="78" max="78" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -7332,14 +7308,14 @@
       <c r="F23" s="65">
         <v>5</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>128</v>
       </c>
       <c r="H23" s="65">
         <f>F23*G23</f>
         <v>1500</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="65">
@@ -7467,20 +7443,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>AN23+AO23+AP23</f>
         <v>279.476</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>215</v>
       </c>
       <c r="AW23" s="66">
@@ -7519,10 +7495,10 @@
       <c r="BL23" s="66" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>221</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>220</v>
       </c>
       <c r="BO23" s="66">
@@ -7546,19 +7522,19 @@
       <c r="BT23" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="BU23" t="s" s="0">
+      <c r="BU23" t="s">
         <v>204</v>
       </c>
-      <c r="BV23" t="s" s="0">
+      <c r="BV23" t="s">
         <v>216</v>
       </c>
-      <c r="BW23" t="s" s="0">
+      <c r="BW23" t="s">
         <v>216</v>
       </c>
-      <c r="BX23" t="s" s="0">
+      <c r="BX23" t="s">
         <v>217</v>
       </c>
-      <c r="BY23" t="s" s="0">
+      <c r="BY23" t="s">
         <v>109</v>
       </c>
       <c r="BZ23" s="97">
@@ -7733,40 +7709,40 @@
   <dimension ref="A1:CC25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="18" max="18" customWidth="true" width="11.28515625"/>
-    <col min="19" max="19" customWidth="true" width="11.140625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="23.85546875"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="50" max="50" customWidth="true" width="11.0"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
-    <col min="78" max="78" bestFit="true" customWidth="true" width="17.5703125"/>
-    <col min="79" max="79" bestFit="true" customWidth="true" width="14.0"/>
-    <col min="81" max="81" bestFit="true" customWidth="true" width="17.28515625"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="18" max="18" width="11.28515625" customWidth="1"/>
+    <col min="19" max="19" width="11.140625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="23.85546875" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="50" max="50" width="11" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="78" max="78" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="79" max="79" width="14" bestFit="1" customWidth="1"/>
+    <col min="81" max="81" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -9328,14 +9304,14 @@
       <c r="F23" s="46">
         <v>5</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>128</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>1500</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -9463,20 +9439,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>279.476</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>215</v>
       </c>
       <c r="AW23" s="48">
@@ -9515,10 +9491,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>223</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>222</v>
       </c>
       <c r="BO23" s="48">
@@ -9542,7 +9518,7 @@
       <c r="BT23" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="BU23" t="s" s="0">
+      <c r="BU23" t="s">
         <v>204</v>
       </c>
       <c r="BV23" s="74" t="s">
@@ -9667,11 +9643,11 @@
       <c r="AQ24" s="56"/>
       <c r="AR24" s="56"/>
       <c r="AS24" s="8"/>
-      <c r="CB24" s="0">
+      <c r="CB24">
         <f>300*U23</f>
         <v>54</v>
       </c>
-      <c r="CC24" s="0">
+      <c r="CC24">
         <f>600*U23</f>
         <v>108</v>
       </c>
@@ -9739,32 +9715,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -11425,20 +11401,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -11477,10 +11453,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>164</v>
       </c>
       <c r="BO23" s="48">
@@ -11655,32 +11631,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -13341,11 +13317,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -13556,34 +13532,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -15109,14 +15085,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -15244,20 +15220,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>189</v>
       </c>
       <c r="AW23" s="48">
@@ -15296,10 +15272,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48">
@@ -15472,32 +15448,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -17023,14 +16999,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -17158,11 +17134,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -17373,34 +17349,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -18926,14 +18902,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -19061,20 +19037,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>158</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>177</v>
       </c>
       <c r="AW23" s="48">
@@ -19113,10 +19089,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>178</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>131</v>
       </c>
       <c r="BO23" s="48">
@@ -19292,32 +19268,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -20843,14 +20819,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -20978,11 +20954,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -21194,34 +21170,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -22747,14 +22723,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -22882,20 +22858,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>132</v>
       </c>
       <c r="AW23" s="48">
@@ -22934,10 +22910,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48">
@@ -23112,44 +23088,44 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="99" width="9.0"/>
-    <col min="2" max="2" customWidth="true" style="99" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" style="99" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" style="99" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" style="99" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" style="99" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" style="99" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" style="99" width="11.85546875"/>
-    <col min="9" max="10" style="99" width="9.0"/>
-    <col min="11" max="11" customWidth="true" style="99" width="6.28515625"/>
-    <col min="12" max="28" style="99" width="9.0"/>
-    <col min="29" max="29" customWidth="true" style="99" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" style="99" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" style="99" width="8.7109375"/>
-    <col min="32" max="34" style="99" width="9.0"/>
-    <col min="35" max="35" customWidth="true" style="99" width="14.28515625"/>
-    <col min="36" max="42" style="99" width="9.0"/>
-    <col min="43" max="43" customWidth="true" style="99" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" style="99" width="23.28515625"/>
-    <col min="45" max="45" style="99" width="9.0"/>
-    <col min="46" max="46" customWidth="true" style="99" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" style="99" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" style="99" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" style="99" width="11.42578125"/>
-    <col min="50" max="50" style="99" width="9.0"/>
-    <col min="51" max="51" customWidth="true" style="99" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" style="99" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" style="99" width="19.0"/>
-    <col min="54" max="59" style="99" width="9.0"/>
-    <col min="60" max="60" customWidth="true" style="99" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" style="99" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" style="99" width="30.5703125"/>
-    <col min="64" max="64" style="99" width="9.0"/>
-    <col min="65" max="65" customWidth="true" style="99" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" style="99" width="37.0"/>
-    <col min="67" max="67" customWidth="true" style="99" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" style="99" width="34.42578125"/>
-    <col min="69" max="16384" style="99" width="9.0"/>
+    <col min="1" max="1" width="9" style="99"/>
+    <col min="2" max="2" width="26.85546875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" style="99" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="99" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="99" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="99" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="99" customWidth="1"/>
+    <col min="9" max="10" width="9" style="99"/>
+    <col min="11" max="11" width="6.28515625" style="99" customWidth="1"/>
+    <col min="12" max="28" width="9" style="99"/>
+    <col min="29" max="29" width="10.28515625" style="99" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" style="99" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="99" customWidth="1"/>
+    <col min="32" max="34" width="9" style="99"/>
+    <col min="35" max="35" width="14.28515625" style="99" customWidth="1"/>
+    <col min="36" max="42" width="9" style="99"/>
+    <col min="43" max="43" width="11.85546875" style="99" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" style="99" customWidth="1"/>
+    <col min="45" max="45" width="9" style="99"/>
+    <col min="46" max="46" width="11.85546875" style="99" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="99" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" style="99" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" style="99" customWidth="1"/>
+    <col min="50" max="50" width="9" style="99"/>
+    <col min="51" max="51" width="13.85546875" style="99" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" style="99" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" style="99" bestFit="1" customWidth="1"/>
+    <col min="54" max="59" width="9" style="99"/>
+    <col min="60" max="60" width="12.5703125" style="99" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" style="99" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" style="99" customWidth="1"/>
+    <col min="64" max="64" width="9" style="99"/>
+    <col min="65" max="65" width="41.140625" style="99" customWidth="1"/>
+    <col min="66" max="66" width="37" style="99" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" style="99" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" style="99" customWidth="1"/>
+    <col min="69" max="16384" width="9" style="99"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -24863,10 +24839,10 @@
         <v>148</v>
       </c>
       <c r="BM23" s="99" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="BN23" s="99" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -24886,10 +24862,10 @@
         <v>2</v>
       </c>
       <c r="B24" s="107" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C24" s="107" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D24" s="157" t="s">
         <v>12</v>
@@ -25088,10 +25064,10 @@
         <v>148</v>
       </c>
       <c r="BM24" s="99" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="BN24" s="99" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="BO24" s="112">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -25262,34 +25238,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -26815,14 +26791,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -26950,20 +26926,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -27002,10 +26978,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -27180,32 +27156,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -28731,14 +28707,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -28866,11 +28842,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -29081,34 +29057,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -30634,14 +30610,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -30769,20 +30745,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>164</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>165</v>
       </c>
       <c r="AW23" s="48">
@@ -30821,10 +30797,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>163</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>127</v>
       </c>
       <c r="BO23" s="48">
@@ -30999,32 +30975,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -32550,14 +32526,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -32685,11 +32661,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -32900,34 +32876,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -34453,14 +34429,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -34588,20 +34564,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>186.32</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>189</v>
       </c>
       <c r="AW23" s="48">
@@ -34640,10 +34616,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>195</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>194</v>
       </c>
       <c r="BO23" s="48">
@@ -34818,32 +34794,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -36369,14 +36345,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -36504,11 +36480,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -36719,34 +36695,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -38407,20 +38383,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>175</v>
       </c>
       <c r="AW23" s="48">
@@ -38459,10 +38435,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>175</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>176</v>
       </c>
       <c r="BO23" s="48">
@@ -38634,34 +38610,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -40322,20 +40298,20 @@
       <c r="AQ23" s="65" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>846.99</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="66" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>175</v>
       </c>
       <c r="AW23" s="48">
@@ -40374,10 +40350,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>175</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>196</v>
       </c>
       <c r="BO23" s="48">
@@ -40549,32 +40525,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -42100,14 +42076,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>162</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>115</v>
       </c>
       <c r="J23" s="46">
@@ -42235,11 +42211,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -42450,34 +42426,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -44003,14 +43979,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -44138,20 +44114,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>570.48</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>191</v>
       </c>
       <c r="AW23" s="16">
@@ -44190,10 +44166,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>198</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>197</v>
       </c>
       <c r="BO23" s="48">
@@ -44365,44 +44341,44 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="99" width="9.0"/>
-    <col min="2" max="2" customWidth="true" style="99" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" style="99" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" style="99" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" style="99" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" style="99" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" style="99" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" style="99" width="11.85546875"/>
-    <col min="9" max="10" style="99" width="9.0"/>
-    <col min="11" max="11" customWidth="true" style="99" width="6.28515625"/>
-    <col min="12" max="28" style="99" width="9.0"/>
-    <col min="29" max="29" customWidth="true" style="99" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" style="99" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" style="99" width="8.7109375"/>
-    <col min="32" max="34" style="99" width="9.0"/>
-    <col min="35" max="35" customWidth="true" style="99" width="14.28515625"/>
-    <col min="36" max="42" style="99" width="9.0"/>
-    <col min="43" max="43" customWidth="true" style="99" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" style="99" width="23.28515625"/>
-    <col min="45" max="45" style="99" width="9.0"/>
-    <col min="46" max="46" customWidth="true" style="99" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" style="99" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" style="99" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" style="99" width="11.42578125"/>
-    <col min="50" max="50" style="99" width="9.0"/>
-    <col min="51" max="51" customWidth="true" style="99" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" style="99" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" style="99" width="19.0"/>
-    <col min="54" max="59" style="99" width="9.0"/>
-    <col min="60" max="60" customWidth="true" style="99" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" style="99" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" style="99" width="30.5703125"/>
-    <col min="64" max="64" bestFit="true" customWidth="true" style="99" width="10.5703125"/>
-    <col min="65" max="65" customWidth="true" style="99" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" style="99" width="37.0"/>
-    <col min="67" max="67" customWidth="true" style="99" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" style="99" width="34.42578125"/>
-    <col min="69" max="16384" style="99" width="9.0"/>
+    <col min="1" max="1" width="9" style="99"/>
+    <col min="2" max="2" width="26.85546875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" style="99" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="99" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="99" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="99" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="99" customWidth="1"/>
+    <col min="9" max="10" width="9" style="99"/>
+    <col min="11" max="11" width="6.28515625" style="99" customWidth="1"/>
+    <col min="12" max="28" width="9" style="99"/>
+    <col min="29" max="29" width="10.28515625" style="99" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" style="99" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="99" customWidth="1"/>
+    <col min="32" max="34" width="9" style="99"/>
+    <col min="35" max="35" width="14.28515625" style="99" customWidth="1"/>
+    <col min="36" max="42" width="9" style="99"/>
+    <col min="43" max="43" width="11.85546875" style="99" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" style="99" customWidth="1"/>
+    <col min="45" max="45" width="9" style="99"/>
+    <col min="46" max="46" width="11.85546875" style="99" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="99" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" style="99" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" style="99" customWidth="1"/>
+    <col min="50" max="50" width="9" style="99"/>
+    <col min="51" max="51" width="13.85546875" style="99" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" style="99" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" style="99" bestFit="1" customWidth="1"/>
+    <col min="54" max="59" width="9" style="99"/>
+    <col min="60" max="60" width="12.5703125" style="99" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" style="99" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" style="99" customWidth="1"/>
+    <col min="64" max="64" width="10.5703125" style="99" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" style="99" customWidth="1"/>
+    <col min="66" max="66" width="37" style="99" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" style="99" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" style="99" customWidth="1"/>
+    <col min="69" max="16384" width="9" style="99"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -46113,13 +46089,13 @@
       <c r="BH23" s="113"/>
       <c r="BI23" s="112"/>
       <c r="BL23" s="112" t="s">
+        <v>231</v>
+      </c>
+      <c r="BM23" s="99" t="s">
         <v>233</v>
       </c>
-      <c r="BM23" s="99" t="s">
-        <v>235</v>
-      </c>
       <c r="BN23" s="99" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -46139,10 +46115,10 @@
         <v>2</v>
       </c>
       <c r="B24" s="107" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C24" s="107" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D24" s="157" t="s">
         <v>12</v>
@@ -46338,13 +46314,13 @@
       <c r="BH24" s="113"/>
       <c r="BI24" s="112"/>
       <c r="BL24" s="112" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="BM24" s="99" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="BN24" s="99" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="BO24" s="112">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -46515,34 +46491,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -48068,14 +48044,14 @@
       <c r="F23" s="46">
         <v>3</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>600</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -48203,20 +48179,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>AN23+AO23+AP23</f>
         <v>558.95000000000005</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>212</v>
       </c>
       <c r="AW23" s="48">
@@ -48255,10 +48231,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>214</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>213</v>
       </c>
       <c r="BO23" s="48">
@@ -48430,32 +48406,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -49981,14 +49957,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -50116,11 +50092,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>188.22</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -50331,34 +50307,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -51884,14 +51860,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -52019,20 +51995,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>564.66</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>191</v>
       </c>
       <c r="AW23" s="16">
@@ -52071,10 +52047,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>191</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>193</v>
       </c>
       <c r="BO23" s="48">
@@ -52249,34 +52225,34 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="36.0"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="36" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -53802,14 +53778,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>400</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -53937,20 +53913,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>564.66</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>191</v>
       </c>
       <c r="AW23" s="16">
@@ -53989,10 +53965,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>191</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>192</v>
       </c>
       <c r="BO23" s="48">
@@ -54167,32 +54143,32 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -55718,14 +55694,14 @@
       <c r="F23" s="46">
         <v>2</v>
       </c>
-      <c r="G23" t="s" s="0">
+      <c r="G23" t="s">
         <v>109</v>
       </c>
       <c r="H23" s="46">
         <f>F23*G23</f>
         <v>40</v>
       </c>
-      <c r="I23" t="s" s="0">
+      <c r="I23" t="s">
         <v>127</v>
       </c>
       <c r="J23" s="46">
@@ -55853,11 +55829,11 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>18.824999999999999</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
@@ -56068,44 +56044,44 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="99" width="9.0"/>
-    <col min="2" max="2" customWidth="true" style="99" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" style="99" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" style="99" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" style="99" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" style="99" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" style="99" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" style="99" width="11.85546875"/>
-    <col min="9" max="10" style="99" width="9.0"/>
-    <col min="11" max="11" customWidth="true" style="99" width="6.28515625"/>
-    <col min="12" max="28" style="99" width="9.0"/>
-    <col min="29" max="29" customWidth="true" style="99" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" style="99" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" style="99" width="8.7109375"/>
-    <col min="32" max="34" style="99" width="9.0"/>
-    <col min="35" max="35" customWidth="true" style="99" width="14.28515625"/>
-    <col min="36" max="42" style="99" width="9.0"/>
-    <col min="43" max="43" customWidth="true" style="99" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" style="99" width="23.28515625"/>
-    <col min="45" max="45" style="99" width="9.0"/>
-    <col min="46" max="46" customWidth="true" style="99" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" style="99" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" style="99" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" style="99" width="11.42578125"/>
-    <col min="50" max="50" style="99" width="9.0"/>
-    <col min="51" max="51" customWidth="true" style="99" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" style="99" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" style="99" width="19.0"/>
-    <col min="54" max="59" style="99" width="9.0"/>
-    <col min="60" max="60" customWidth="true" style="99" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" style="99" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" style="99" width="30.5703125"/>
-    <col min="64" max="64" bestFit="true" customWidth="true" style="99" width="10.5703125"/>
-    <col min="65" max="65" customWidth="true" style="99" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" style="99" width="37.0"/>
-    <col min="67" max="67" customWidth="true" style="99" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" style="99" width="34.42578125"/>
-    <col min="69" max="16384" style="99" width="9.0"/>
+    <col min="1" max="1" width="9" style="99"/>
+    <col min="2" max="2" width="26.85546875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" style="99" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="99" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="99" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="99" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="99" customWidth="1"/>
+    <col min="9" max="10" width="9" style="99"/>
+    <col min="11" max="11" width="6.28515625" style="99" customWidth="1"/>
+    <col min="12" max="28" width="9" style="99"/>
+    <col min="29" max="29" width="10.28515625" style="99" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" style="99" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="99" customWidth="1"/>
+    <col min="32" max="34" width="9" style="99"/>
+    <col min="35" max="35" width="14.28515625" style="99" customWidth="1"/>
+    <col min="36" max="42" width="9" style="99"/>
+    <col min="43" max="43" width="11.85546875" style="99" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" style="99" customWidth="1"/>
+    <col min="45" max="45" width="9" style="99"/>
+    <col min="46" max="46" width="11.85546875" style="99" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="99" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" style="99" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" style="99" customWidth="1"/>
+    <col min="50" max="50" width="9" style="99"/>
+    <col min="51" max="51" width="13.85546875" style="99" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" style="99" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" style="99" bestFit="1" customWidth="1"/>
+    <col min="54" max="59" width="9" style="99"/>
+    <col min="60" max="60" width="12.5703125" style="99" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" style="99" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" style="99" customWidth="1"/>
+    <col min="64" max="64" width="10.5703125" style="99" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" style="99" customWidth="1"/>
+    <col min="66" max="66" width="37" style="99" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" style="99" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" style="99" customWidth="1"/>
+    <col min="69" max="16384" width="9" style="99"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -57816,10 +57792,10 @@
       <c r="BH23" s="113"/>
       <c r="BI23" s="112"/>
       <c r="BL23" s="112" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="BM23" s="99" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="BN23" s="99" t="s">
         <v>173</v>
@@ -57993,44 +57969,44 @@
   <dimension ref="A1:BR26"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="99" width="9.0"/>
-    <col min="2" max="2" customWidth="true" style="99" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" style="99" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" style="99" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" style="99" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" style="99" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" style="99" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" style="99" width="11.85546875"/>
-    <col min="9" max="10" style="99" width="9.0"/>
-    <col min="11" max="11" customWidth="true" style="99" width="6.28515625"/>
-    <col min="12" max="28" style="99" width="9.0"/>
-    <col min="29" max="29" customWidth="true" style="99" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" style="99" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" style="99" width="8.7109375"/>
-    <col min="32" max="34" style="99" width="9.0"/>
-    <col min="35" max="35" customWidth="true" style="99" width="14.28515625"/>
-    <col min="36" max="42" style="99" width="9.0"/>
-    <col min="43" max="43" customWidth="true" style="99" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" style="99" width="23.28515625"/>
-    <col min="45" max="45" style="99" width="9.0"/>
-    <col min="46" max="46" customWidth="true" style="99" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" style="99" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" style="99" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" style="99" width="11.42578125"/>
-    <col min="50" max="50" style="99" width="9.0"/>
-    <col min="51" max="51" customWidth="true" style="99" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" style="99" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" style="99" width="19.0"/>
-    <col min="54" max="59" style="99" width="9.0"/>
-    <col min="60" max="60" customWidth="true" style="99" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" style="99" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" style="99" width="30.5703125"/>
-    <col min="64" max="64" style="99" width="9.0"/>
-    <col min="65" max="65" customWidth="true" style="99" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" style="99" width="37.0"/>
-    <col min="67" max="67" customWidth="true" style="99" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" style="99" width="34.42578125"/>
-    <col min="69" max="16384" style="99" width="9.0"/>
+    <col min="1" max="1" width="9" style="99"/>
+    <col min="2" max="2" width="26.85546875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" style="99" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="99" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="99" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="99" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="99" customWidth="1"/>
+    <col min="9" max="10" width="9" style="99"/>
+    <col min="11" max="11" width="6.28515625" style="99" customWidth="1"/>
+    <col min="12" max="28" width="9" style="99"/>
+    <col min="29" max="29" width="10.28515625" style="99" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" style="99" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="99" customWidth="1"/>
+    <col min="32" max="34" width="9" style="99"/>
+    <col min="35" max="35" width="14.28515625" style="99" customWidth="1"/>
+    <col min="36" max="42" width="9" style="99"/>
+    <col min="43" max="43" width="11.85546875" style="99" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" style="99" customWidth="1"/>
+    <col min="45" max="45" width="9" style="99"/>
+    <col min="46" max="46" width="11.85546875" style="99" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="99" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" style="99" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" style="99" customWidth="1"/>
+    <col min="50" max="50" width="9" style="99"/>
+    <col min="51" max="51" width="13.85546875" style="99" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" style="99" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" style="99" bestFit="1" customWidth="1"/>
+    <col min="54" max="59" width="9" style="99"/>
+    <col min="60" max="60" width="12.5703125" style="99" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" style="99" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" style="99" customWidth="1"/>
+    <col min="64" max="64" width="9" style="99"/>
+    <col min="65" max="65" width="41.140625" style="99" customWidth="1"/>
+    <col min="66" max="66" width="37" style="99" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" style="99" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" style="99" customWidth="1"/>
+    <col min="69" max="16384" width="9" style="99"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -59705,7 +59681,7 @@
         <v>108</v>
       </c>
       <c r="AV23" s="99" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="AW23" s="112">
         <f>AM23</f>
@@ -59744,10 +59720,10 @@
         <v>148</v>
       </c>
       <c r="BM23" s="99" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="BN23" s="99" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -59767,10 +59743,10 @@
         <v>2</v>
       </c>
       <c r="B24" s="107" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C24" s="107" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D24" s="157" t="s">
         <v>12</v>
@@ -59930,7 +59906,7 @@
         <v>108</v>
       </c>
       <c r="AV24" s="99" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="AW24" s="112">
         <f>AM24</f>
@@ -59969,10 +59945,10 @@
         <v>148</v>
       </c>
       <c r="BM24" s="99" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="BN24" s="99" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="BO24" s="112">
         <f>ROUND((((AW24*AZ24)+(BN24*BM24))/(AW24+BN24)),5)</f>
@@ -60143,44 +60119,44 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" style="99" width="9.0"/>
-    <col min="2" max="2" customWidth="true" style="99" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" style="99" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" style="99" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" style="99" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" style="99" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" style="99" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" style="99" width="11.85546875"/>
-    <col min="9" max="10" style="99" width="9.0"/>
-    <col min="11" max="11" customWidth="true" style="99" width="6.28515625"/>
-    <col min="12" max="28" style="99" width="9.0"/>
-    <col min="29" max="29" customWidth="true" style="99" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" style="99" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" style="99" width="8.7109375"/>
-    <col min="32" max="34" style="99" width="9.0"/>
-    <col min="35" max="35" customWidth="true" style="99" width="14.28515625"/>
-    <col min="36" max="42" style="99" width="9.0"/>
-    <col min="43" max="43" customWidth="true" style="99" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" style="99" width="23.28515625"/>
-    <col min="45" max="45" style="99" width="9.0"/>
-    <col min="46" max="46" customWidth="true" style="99" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" style="99" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" style="99" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" style="99" width="11.42578125"/>
-    <col min="50" max="50" style="99" width="9.0"/>
-    <col min="51" max="51" customWidth="true" style="99" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" style="99" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" style="99" width="19.0"/>
-    <col min="54" max="59" style="99" width="9.0"/>
-    <col min="60" max="60" customWidth="true" style="99" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" style="99" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" style="99" width="30.5703125"/>
-    <col min="64" max="64" style="99" width="9.0"/>
-    <col min="65" max="65" customWidth="true" style="99" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" style="99" width="37.0"/>
-    <col min="67" max="67" customWidth="true" style="99" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" style="99" width="34.42578125"/>
-    <col min="69" max="16384" style="99" width="9.0"/>
+    <col min="1" max="1" width="9" style="99"/>
+    <col min="2" max="2" width="26.85546875" style="99" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="99" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" style="99" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="99" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" style="99" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" style="99" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" style="99" customWidth="1"/>
+    <col min="9" max="10" width="9" style="99"/>
+    <col min="11" max="11" width="6.28515625" style="99" customWidth="1"/>
+    <col min="12" max="28" width="9" style="99"/>
+    <col min="29" max="29" width="10.28515625" style="99" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" style="99" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" style="99" customWidth="1"/>
+    <col min="32" max="34" width="9" style="99"/>
+    <col min="35" max="35" width="14.28515625" style="99" customWidth="1"/>
+    <col min="36" max="42" width="9" style="99"/>
+    <col min="43" max="43" width="11.85546875" style="99" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" style="99" customWidth="1"/>
+    <col min="45" max="45" width="9" style="99"/>
+    <col min="46" max="46" width="11.85546875" style="99" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" style="99" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" style="99" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" style="99" customWidth="1"/>
+    <col min="50" max="50" width="9" style="99"/>
+    <col min="51" max="51" width="13.85546875" style="99" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" style="99" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" style="99" bestFit="1" customWidth="1"/>
+    <col min="54" max="59" width="9" style="99"/>
+    <col min="60" max="60" width="12.5703125" style="99" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" style="99" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" style="99" customWidth="1"/>
+    <col min="64" max="64" width="9" style="99"/>
+    <col min="65" max="65" width="41.140625" style="99" customWidth="1"/>
+    <col min="66" max="66" width="37" style="99" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" style="99" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" style="99" customWidth="1"/>
+    <col min="69" max="16384" width="9" style="99"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -61851,11 +61827,11 @@
       <c r="AT23" s="112" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="99">
+      <c r="AU23" s="99" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="99">
-        <v>242</v>
+      <c r="AV23" s="99" t="s">
+        <v>240</v>
       </c>
       <c r="AW23" s="112">
         <f>AM23</f>
@@ -61893,11 +61869,11 @@
       <c r="BL23" s="112" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="99">
-        <v>250</v>
-      </c>
-      <c r="BN23" t="s" s="99">
-        <v>249</v>
+      <c r="BM23" s="99" t="s">
+        <v>242</v>
+      </c>
+      <c r="BN23" s="99" t="s">
+        <v>241</v>
       </c>
       <c r="BO23" s="112">
         <f>ROUND((((AW23*AZ23)+(BN23*BM23))/(AW23+BN23)),5)</f>
@@ -62068,7 +62044,7 @@
   <dimension ref="A8:BR37"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="27.28515625"/>
+    <col min="2" max="2" width="27.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="8" spans="1:70" ht="15.75" thickBot="1"/>
@@ -62236,10 +62212,10 @@
       <c r="AT9" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU9" t="s" s="0">
+      <c r="AU9" t="s">
         <v>127</v>
       </c>
-      <c r="AV9" t="s" s="0">
+      <c r="AV9" t="s">
         <v>143</v>
       </c>
       <c r="AW9" s="48">
@@ -62280,10 +62256,10 @@
       <c r="BL9" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM9" t="s" s="0">
+      <c r="BM9" t="s">
         <v>146</v>
       </c>
-      <c r="BN9" t="s" s="0">
+      <c r="BN9" t="s">
         <v>147</v>
       </c>
       <c r="BO9" s="48" t="e">
@@ -62455,20 +62431,20 @@
       <c r="AQ15" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR15" t="e" s="0">
+      <c r="AR15" t="e">
         <f>ROUND(AN15+AO15+AP15,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS15" t="s" s="0">
+      <c r="AS15" t="s">
         <v>107</v>
       </c>
       <c r="AT15" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU15" t="s" s="0">
+      <c r="AU15" t="s">
         <v>131</v>
       </c>
-      <c r="AV15" t="s" s="0">
+      <c r="AV15" t="s">
         <v>149</v>
       </c>
       <c r="AW15" s="48">
@@ -62507,10 +62483,10 @@
       <c r="BL15" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM15" t="s" s="0">
+      <c r="BM15" t="s">
         <v>149</v>
       </c>
-      <c r="BN15" t="s" s="0">
+      <c r="BN15" t="s">
         <v>150</v>
       </c>
       <c r="BO15" s="48" t="e">
@@ -62680,20 +62656,20 @@
       <c r="AQ16" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR16" s="0">
+      <c r="AR16">
         <f>ROUND(AN16+AO16+AP16,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS16" t="s" s="0">
+      <c r="AS16" t="s">
         <v>107</v>
       </c>
       <c r="AT16" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU16" t="s" s="0">
+      <c r="AU16" t="s">
         <v>135</v>
       </c>
-      <c r="AV16" t="s" s="0">
+      <c r="AV16" t="s">
         <v>136</v>
       </c>
       <c r="AW16" s="48">
@@ -62732,10 +62708,10 @@
       <c r="BL16" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM16" t="s" s="0">
+      <c r="BM16" t="s">
         <v>134</v>
       </c>
-      <c r="BN16" t="s" s="0">
+      <c r="BN16" t="s">
         <v>133</v>
       </c>
       <c r="BO16" s="48">
@@ -62905,20 +62881,20 @@
       <c r="AQ17" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR17" s="0">
+      <c r="AR17">
         <f>ROUND(AN17+AO17+AP17,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS17" t="s" s="0">
+      <c r="AS17" t="s">
         <v>107</v>
       </c>
       <c r="AT17" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU17" t="s" s="0">
+      <c r="AU17" t="s">
         <v>108</v>
       </c>
-      <c r="AV17" t="s" s="0">
+      <c r="AV17" t="s">
         <v>132</v>
       </c>
       <c r="AW17" s="48">
@@ -63124,20 +63100,20 @@
       <c r="AQ18" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR18" s="0">
+      <c r="AR18">
         <f>ROUND(AN18+AO18+AP18,5)</f>
         <v>234.33</v>
       </c>
-      <c r="AS18" t="s" s="0">
+      <c r="AS18" t="s">
         <v>107</v>
       </c>
       <c r="AT18" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU18" t="s" s="0">
+      <c r="AU18" t="s">
         <v>130</v>
       </c>
-      <c r="AV18" t="s" s="0">
+      <c r="AV18" t="s">
         <v>137</v>
       </c>
       <c r="AW18" s="48">
@@ -63176,10 +63152,10 @@
       <c r="BL18" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="BM18" t="s" s="0">
+      <c r="BM18" t="s">
         <v>153</v>
       </c>
-      <c r="BN18" t="s" s="0">
+      <c r="BN18" t="s">
         <v>152</v>
       </c>
       <c r="BO18" s="48">
@@ -63350,20 +63326,20 @@
       <c r="AQ20" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR20" t="e" s="0">
+      <c r="AR20" t="e">
         <f>ROUND(AN20+AO20+AP20,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS20" t="s" s="0">
+      <c r="AS20" t="s">
         <v>107</v>
       </c>
       <c r="AT20" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU20" t="s" s="0">
+      <c r="AU20" t="s">
         <v>155</v>
       </c>
-      <c r="AV20" t="s" s="0">
+      <c r="AV20" t="s">
         <v>156</v>
       </c>
       <c r="AW20" s="48">
@@ -63402,10 +63378,10 @@
       <c r="BL20" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM20" t="s" s="0">
+      <c r="BM20" t="s">
         <v>156</v>
       </c>
-      <c r="BN20" t="s" s="0">
+      <c r="BN20" t="s">
         <v>127</v>
       </c>
       <c r="BO20" s="48" t="e">
@@ -63575,20 +63551,20 @@
       <c r="AQ21" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR21" t="e" s="0">
+      <c r="AR21" t="e">
         <f t="shared" ref="AR21:AR23" si="30">ROUND(AN21+AO21+AP21,5)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS21" t="s" s="0">
+      <c r="AS21" t="s">
         <v>107</v>
       </c>
       <c r="AT21" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU21" t="s" s="0">
+      <c r="AU21" t="s">
         <v>131</v>
       </c>
-      <c r="AV21" t="s" s="0">
+      <c r="AV21" t="s">
         <v>157</v>
       </c>
       <c r="AW21" s="48">
@@ -63627,10 +63603,10 @@
       <c r="BL21" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM21" t="s" s="0">
+      <c r="BM21" t="s">
         <v>108</v>
       </c>
-      <c r="BN21" t="s" s="0">
+      <c r="BN21" t="s">
         <v>108</v>
       </c>
       <c r="BO21" s="48" t="e">
@@ -63800,20 +63776,20 @@
       <c r="AQ22" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR22" t="e" s="0">
+      <c r="AR22" t="e">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS22" t="s" s="0">
+      <c r="AS22" t="s">
         <v>107</v>
       </c>
       <c r="AT22" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU22" t="s" s="0">
+      <c r="AU22" t="s">
         <v>158</v>
       </c>
-      <c r="AV22" t="s" s="0">
+      <c r="AV22" t="s">
         <v>159</v>
       </c>
       <c r="AW22" s="48">
@@ -63852,10 +63828,10 @@
       <c r="BL22" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM22" t="s" s="0">
+      <c r="BM22" t="s">
         <v>108</v>
       </c>
-      <c r="BN22" t="s" s="0">
+      <c r="BN22" t="s">
         <v>108</v>
       </c>
       <c r="BO22" s="48" t="e">
@@ -64025,20 +64001,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" t="e" s="0">
+      <c r="AR23" t="e">
         <f t="shared" si="30"/>
         <v>#DIV/0!</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>107</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>160</v>
       </c>
       <c r="AW23" s="48">
@@ -64077,10 +64053,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>108</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>108</v>
       </c>
       <c r="BO23" s="48" t="e">
@@ -64137,14 +64113,14 @@
       <c r="F31" s="46">
         <v>2</v>
       </c>
-      <c r="G31" t="s" s="0">
+      <c r="G31" t="s">
         <v>128</v>
       </c>
       <c r="H31" s="46">
         <f>F31*G31</f>
         <v>600</v>
       </c>
-      <c r="I31" t="s" s="0">
+      <c r="I31" t="s">
         <v>127</v>
       </c>
       <c r="J31" s="46">
@@ -64272,20 +64248,20 @@
       <c r="AQ31" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR31" s="0">
+      <c r="AR31">
         <f>ROUND(AN31+AO31+AP31,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS31" t="s" s="0">
+      <c r="AS31" t="s">
         <v>107</v>
       </c>
       <c r="AT31" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU31" t="s" s="0">
+      <c r="AU31" t="s">
         <v>162</v>
       </c>
-      <c r="AV31" t="s" s="0">
+      <c r="AV31" t="s">
         <v>167</v>
       </c>
       <c r="AW31" s="48">
@@ -64324,10 +64300,10 @@
       <c r="BL31" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM31" t="s" s="0">
+      <c r="BM31" t="s">
         <v>108</v>
       </c>
-      <c r="BN31" t="s" s="0">
+      <c r="BN31" t="s">
         <v>108</v>
       </c>
       <c r="BO31" s="48">
@@ -64362,14 +64338,14 @@
       <c r="F32" s="46">
         <v>2</v>
       </c>
-      <c r="G32" t="s" s="0">
+      <c r="G32" t="s">
         <v>129</v>
       </c>
       <c r="H32" s="46">
         <f>F32*G32</f>
         <v>800</v>
       </c>
-      <c r="I32" t="s" s="0">
+      <c r="I32" t="s">
         <v>127</v>
       </c>
       <c r="J32" s="46">
@@ -64497,20 +64473,20 @@
       <c r="AQ32" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR32" s="0">
+      <c r="AR32">
         <f>ROUND(AN32+AO32+AP32,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS32" t="s" s="0">
+      <c r="AS32" t="s">
         <v>107</v>
       </c>
       <c r="AT32" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU32" t="s" s="0">
+      <c r="AU32" t="s">
         <v>168</v>
       </c>
-      <c r="AV32" t="s" s="0">
+      <c r="AV32" t="s">
         <v>169</v>
       </c>
       <c r="AW32" s="48">
@@ -64549,10 +64525,10 @@
       <c r="BL32" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM32" t="s" s="0">
+      <c r="BM32" t="s">
         <v>108</v>
       </c>
-      <c r="BN32" t="s" s="0">
+      <c r="BN32" t="s">
         <v>108</v>
       </c>
       <c r="BO32" s="48">
@@ -64587,14 +64563,14 @@
       <c r="F33" s="46">
         <v>2</v>
       </c>
-      <c r="G33" t="s" s="0">
+      <c r="G33" t="s">
         <v>161</v>
       </c>
       <c r="H33" s="46">
         <f>F33*G33</f>
         <v>1000</v>
       </c>
-      <c r="I33" t="s" s="0">
+      <c r="I33" t="s">
         <v>127</v>
       </c>
       <c r="J33" s="46">
@@ -64722,20 +64698,20 @@
       <c r="AQ33" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR33" s="0">
+      <c r="AR33">
         <f>ROUND(AN33+AO33+AP33,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS33" t="s" s="0">
+      <c r="AS33" t="s">
         <v>107</v>
       </c>
       <c r="AT33" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU33" t="s" s="0">
+      <c r="AU33" t="s">
         <v>108</v>
       </c>
-      <c r="AV33" t="s" s="0">
+      <c r="AV33" t="s">
         <v>170</v>
       </c>
       <c r="AW33" s="48">
@@ -64774,10 +64750,10 @@
       <c r="BL33" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM33" t="s" s="0">
+      <c r="BM33" t="s">
         <v>108</v>
       </c>
-      <c r="BN33" t="s" s="0">
+      <c r="BN33" t="s">
         <v>108</v>
       </c>
       <c r="BO33" s="48">
@@ -64813,14 +64789,14 @@
       <c r="F35" s="46">
         <v>2</v>
       </c>
-      <c r="G35" t="s" s="0">
+      <c r="G35" t="s">
         <v>128</v>
       </c>
       <c r="H35" s="46">
         <f>F35*G35</f>
         <v>600</v>
       </c>
-      <c r="I35" t="s" s="0">
+      <c r="I35" t="s">
         <v>127</v>
       </c>
       <c r="J35" s="46">
@@ -64948,20 +64924,20 @@
       <c r="AQ35" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR35" s="0">
+      <c r="AR35">
         <f>ROUND(AN35+AO35+AP35,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS35" t="s" s="0">
+      <c r="AS35" t="s">
         <v>107</v>
       </c>
       <c r="AT35" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU35" t="s" s="0">
+      <c r="AU35" t="s">
         <v>171</v>
       </c>
-      <c r="AV35" t="s" s="0">
+      <c r="AV35" t="s">
         <v>172</v>
       </c>
       <c r="AW35" s="48">
@@ -65000,10 +64976,10 @@
       <c r="BL35" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM35" t="s" s="0">
+      <c r="BM35" t="s">
         <v>108</v>
       </c>
-      <c r="BN35" t="s" s="0">
+      <c r="BN35" t="s">
         <v>108</v>
       </c>
       <c r="BO35" s="48">
@@ -65038,14 +65014,14 @@
       <c r="F36" s="46">
         <v>2</v>
       </c>
-      <c r="G36" t="s" s="0">
+      <c r="G36" t="s">
         <v>129</v>
       </c>
       <c r="H36" s="46">
         <f>F36*G36</f>
         <v>800</v>
       </c>
-      <c r="I36" t="s" s="0">
+      <c r="I36" t="s">
         <v>127</v>
       </c>
       <c r="J36" s="46">
@@ -65173,20 +65149,20 @@
       <c r="AQ36" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR36" s="0">
+      <c r="AR36">
         <f>ROUND(AN36+AO36+AP36,5)</f>
         <v>372.63499999999999</v>
       </c>
-      <c r="AS36" t="s" s="0">
+      <c r="AS36" t="s">
         <v>107</v>
       </c>
       <c r="AT36" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU36" t="s" s="0">
+      <c r="AU36" t="s">
         <v>173</v>
       </c>
-      <c r="AV36" t="s" s="0">
+      <c r="AV36" t="s">
         <v>174</v>
       </c>
       <c r="AW36" s="48">
@@ -65225,10 +65201,10 @@
       <c r="BL36" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM36" t="s" s="0">
+      <c r="BM36" t="s">
         <v>108</v>
       </c>
-      <c r="BN36" t="s" s="0">
+      <c r="BN36" t="s">
         <v>108</v>
       </c>
       <c r="BO36" s="48">
@@ -65263,14 +65239,14 @@
       <c r="F37" s="46">
         <v>2</v>
       </c>
-      <c r="G37" t="s" s="0">
+      <c r="G37" t="s">
         <v>161</v>
       </c>
       <c r="H37" s="46">
         <f>F37*G37</f>
         <v>1000</v>
       </c>
-      <c r="I37" t="s" s="0">
+      <c r="I37" t="s">
         <v>127</v>
       </c>
       <c r="J37" s="46">
@@ -65398,20 +65374,20 @@
       <c r="AQ37" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR37" s="0">
+      <c r="AR37">
         <f>ROUND(AN37+AO37+AP37,5)</f>
         <v>465.79500000000002</v>
       </c>
-      <c r="AS37" t="s" s="0">
+      <c r="AS37" t="s">
         <v>107</v>
       </c>
       <c r="AT37" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU37" t="s" s="0">
+      <c r="AU37" t="s">
         <v>108</v>
       </c>
-      <c r="AV37" t="s" s="0">
+      <c r="AV37" t="s">
         <v>170</v>
       </c>
       <c r="AW37" s="48">
@@ -65450,10 +65426,10 @@
       <c r="BL37" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM37" t="s" s="0">
+      <c r="BM37" t="s">
         <v>108</v>
       </c>
-      <c r="BN37" t="s" s="0">
+      <c r="BN37" t="s">
         <v>108</v>
       </c>
       <c r="BO37" s="48">
@@ -65479,34 +65455,34 @@
   <dimension ref="A1:BR25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -67167,20 +67143,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>282.33</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -67219,10 +67195,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" t="s" s="0">
+      <c r="BM23" t="s">
         <v>149</v>
       </c>
-      <c r="BN23" t="s" s="0">
+      <c r="BN23" t="s">
         <v>155</v>
       </c>
       <c r="BO23" s="48">
@@ -67395,36 +67371,36 @@
   <dimension ref="A1:BU25"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" customWidth="true" width="26.85546875"/>
-    <col min="3" max="3" customWidth="true" width="19.28515625"/>
-    <col min="4" max="4" customWidth="true" width="80.42578125"/>
-    <col min="5" max="5" customWidth="true" width="10.42578125"/>
-    <col min="6" max="6" customWidth="true" width="8.28515625"/>
-    <col min="7" max="7" customWidth="true" width="10.140625"/>
-    <col min="8" max="8" customWidth="true" width="11.85546875"/>
-    <col min="11" max="11" customWidth="true" width="6.28515625"/>
-    <col min="18" max="18" customWidth="true" width="14.85546875"/>
-    <col min="29" max="29" customWidth="true" width="10.28515625"/>
-    <col min="30" max="30" customWidth="true" width="12.85546875"/>
-    <col min="31" max="31" customWidth="true" width="8.7109375"/>
-    <col min="35" max="35" customWidth="true" width="14.28515625"/>
-    <col min="43" max="43" customWidth="true" width="11.85546875"/>
-    <col min="44" max="44" customWidth="true" width="23.28515625"/>
-    <col min="46" max="46" customWidth="true" width="11.85546875"/>
-    <col min="47" max="47" customWidth="true" width="15.28515625"/>
-    <col min="48" max="48" customWidth="true" width="20.28515625"/>
-    <col min="49" max="49" customWidth="true" width="11.42578125"/>
-    <col min="51" max="51" customWidth="true" width="13.85546875"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="18.85546875"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="60" max="60" customWidth="true" width="12.5703125"/>
-    <col min="61" max="61" customWidth="true" width="21.7109375"/>
-    <col min="62" max="63" customWidth="true" width="30.5703125"/>
-    <col min="65" max="65" customWidth="true" width="41.140625"/>
-    <col min="66" max="66" customWidth="true" width="37.0"/>
-    <col min="67" max="67" customWidth="true" width="18.85546875"/>
-    <col min="68" max="68" customWidth="true" width="34.42578125"/>
-    <col min="71" max="71" customWidth="true" width="22.140625"/>
+    <col min="2" max="2" width="26.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="80.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" customWidth="1"/>
+    <col min="7" max="7" width="10.140625" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="11" max="11" width="6.28515625" customWidth="1"/>
+    <col min="18" max="18" width="14.85546875" customWidth="1"/>
+    <col min="29" max="29" width="10.28515625" customWidth="1"/>
+    <col min="30" max="30" width="12.85546875" customWidth="1"/>
+    <col min="31" max="31" width="8.7109375" customWidth="1"/>
+    <col min="35" max="35" width="14.28515625" customWidth="1"/>
+    <col min="43" max="43" width="11.85546875" customWidth="1"/>
+    <col min="44" max="44" width="23.28515625" customWidth="1"/>
+    <col min="46" max="46" width="11.85546875" customWidth="1"/>
+    <col min="47" max="47" width="15.28515625" customWidth="1"/>
+    <col min="48" max="48" width="20.28515625" customWidth="1"/>
+    <col min="49" max="49" width="11.42578125" customWidth="1"/>
+    <col min="51" max="51" width="13.85546875" customWidth="1"/>
+    <col min="52" max="52" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="19" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="12.5703125" customWidth="1"/>
+    <col min="61" max="61" width="21.7109375" customWidth="1"/>
+    <col min="62" max="63" width="30.5703125" customWidth="1"/>
+    <col min="65" max="65" width="41.140625" customWidth="1"/>
+    <col min="66" max="66" width="37" customWidth="1"/>
+    <col min="67" max="67" width="18.85546875" customWidth="1"/>
+    <col min="68" max="68" width="34.42578125" customWidth="1"/>
+    <col min="71" max="71" width="22.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:45" ht="18">
@@ -69097,20 +69073,20 @@
       <c r="AQ23" s="46" t="s">
         <v>12</v>
       </c>
-      <c r="AR23" s="0">
+      <c r="AR23">
         <f>ROUND(AN23+AO23+AP23,5)</f>
         <v>279.47500000000002</v>
       </c>
-      <c r="AS23" t="s" s="0">
+      <c r="AS23" t="s">
         <v>188</v>
       </c>
       <c r="AT23" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="AU23" t="s" s="0">
+      <c r="AU23" t="s">
         <v>108</v>
       </c>
-      <c r="AV23" t="s" s="0">
+      <c r="AV23" t="s">
         <v>149</v>
       </c>
       <c r="AW23" s="48">
@@ -69149,10 +69125,10 @@
       <c r="BL23" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="BM23" s="0">
+      <c r="BM23">
         <v>292.60462000000001</v>
       </c>
-      <c r="BN23" s="0">
+      <c r="BN23">
         <v>682</v>
       </c>
       <c r="BO23" s="48">
@@ -69176,7 +69152,7 @@
       <c r="BT23" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="BU23" t="s" s="0">
+      <c r="BU23" t="s">
         <v>204</v>
       </c>
     </row>

</xml_diff>